<commit_message>
Update Data Dictionary with NCH Homoeopathy dataset (116 fields, 12 datasets)
</commit_message>
<xml_diff>
--- a/DATA_DICTIONARY.xlsx
+++ b/DATA_DICTIONARY.xlsx
@@ -19,7 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBSE_Schools" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CISCE_Schools" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telangana_Census" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Calculated" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NCH_Homoeopathy" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Calculated" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -530,12 +531,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -1171,53 +1172,108 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Homoeopathy Education (BHMS / MD Homoeopathy)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>299</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>26 / 36 (72%)</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>NCH_College_Code (MARBH Assigned)</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Medical Assessment and Rating Board for Homoeopathy (MARBH) Permission Status Roster</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>100% complete national census of recognized/permitted and denied homoeopathic medical colleges across India under NCH Act, 2020.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Cross-Cutting Metadata &amp; Search</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>7,335 Final Records</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>36 / 36 (100%)</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>N/A (Derived Attributes)</t>
         </is>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="I16" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>Pan-India Data Quality &amp; Deduplication Engine</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Standardized canonical state, inferred district, quality status, and search blobs.</t>
         </is>
@@ -2212,6 +2268,878 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DATA DICTIONARY: NCH HOMOEOPATHY COLLEGES REGISTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Field / Column Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Field Classification</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Required?</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Example Value</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Allowed Values / Codebook</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Description / Meaning</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Methodological Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>S.No (NCH)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Sequential serial number (1–299)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Gazetted institution serial number from the official NCH AY 2026-27 permission status document.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>100% sequential across all 25 pages with zero gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Institution Name</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Allu Ramalingaiah Government Homoeopathic Medical College</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Official registered homoeopathic college title</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Standardized, deduplicated official name of the homoeopathic institution, parsed cleanly from the composite header address text.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>100% populated. No missing college names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Full Name &amp; Address</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Allu Ramalingaiah Govt. Homoeo Medical College, D.No. 26-1-11, V.L. Puram, Rajahmundry-533103, East Godavari Distt.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Verbatim institution address and locality string</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Raw unparsed text string from NCH PDF containing college name, postal address, street, district, PIN code, and contact information.</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Primary source textual record for institutional entity verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>arghmcrjy@gmail.com</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Valid email address or empty</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Administrative or institutional principal contact email address parsed from the composite address block using regex pattern matching.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Extracted where present in official directory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Pincode</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>533103</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>6-digit Indian PIN code</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Six-digit postal index number extracted from the campus address block.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Extracted with boundary validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>State/UT</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Standard 36 States/UTs</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>State or Union Territory heading under which the homoeopathic college is officially registered by NCH.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Covers 26 States and UTs offering recognized homoeopathic medical education.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>NCH College Code</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Yes (Where Assigned)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Official MARBH/NCH numeric or alphanumeric college code</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Statutory regulatory identifier assigned to the college by the Medical Assessment and Rating Board for Homoeopathy (MARBH).</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Official regulatory ID. 9 newly applied colleges lack pre-assigned codes and use deterministic canonical keys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Identifier Type</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>NCH_COLLEGE_CODE</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>NCH_COLLEGE_CODE, NCH_DERIVED_KEY</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Audit classification indicating whether the college possesses an official MARBH code or a synthetic deterministic surrogate identifier.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Provides transparency on regulatory ID presence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Canonical Key</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>NCH_101</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>NCH_&lt;CODE&gt; or NCH_DERIVED_&lt;SNO&gt;</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Normalized, immutable institutional key used for national multi-source cross-registry linking.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Ensures unique index representation in master census.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Management Type</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Govt.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Govt., Pvt. (Private), Trust, Society, Grant-in-aid</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Institutional governance and ownership model (Government vs Private/Trust).</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Normalized from raw 'Govt/Pvt' PDF column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>UG Seat Intake</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Numeric seat capacity or 'Nil' / '-'</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Undergraduate Bachelor of Homoeopathic Medicine and Surgery (BHMS) annual student admission intake capacity applied for or permitted.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Applicable for UG-granting institutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>UG Permission</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Numeric permitted seats (including EWS quota) or '-'</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Number of undergraduate BHMS seats officially approved and permitted by MARBH for the academic session 2026-27.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Zero or '-' indicates admission denial or withheld status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>PG Seat Intake</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Numeric seat capacity or '-'</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Postgraduate MD (Homoeopathy) student intake capacity applied for or recognized.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Applicable for PG specialty colleges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>PG Permission</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Numeric permitted PG seats or '-'</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Total postgraduate seats approved by MARBH across clinical and non-clinical homoeopathic disciplines for AY 2026-27.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Subject-wise allocations detailed in companion column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>MARBH Decision</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Conditional Permission</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Permission, Conditional Permission, Denial, Permission Withheld, Status Not Available</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Official regulatory determination issued by the Medical Assessment and Rating Board for Homoeopathy regarding college inspection and compliance.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Key statutory quality indicator governing student admissions for 2026-27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Overall Permission Status</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Conditional Permission</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Conditional Permission (93), Status Not Available (114), Permission (52), Denial (39), Permission Withheld (1)</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Normalized categorical status representing the institution's operational approval standing.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Enables executive filtering and quality dashboard visualization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Scheme</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>UG &amp; PG</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>UG, PG, UG &amp; PG</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Educational program tier authorized at the institution (Undergraduate, Postgraduate, or Both).</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Delineates institutional scope of medical training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Academic Year</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Academic cycle for which the statutory permission status and seat intake quota apply.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Current active AY under MARBH/NCH Gazette.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>URL (String)</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>https://nch.org.in/upload/Permission-Status%20as%20on%2003-08-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Valid HTTPS URL on official nch.org.in portal</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Direct canonical link to the official regulatory PDF document published on the NCH portal.</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Ensures complete data auditability and statutory lineage.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2496,7 +3424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K98"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -2505,7 +3433,7 @@
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="29" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
     <col width="48" customWidth="1" min="9" max="9"/>
     <col width="48" customWidth="1" min="10" max="10"/>
@@ -7816,32 +8744,32 @@
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NCH Homoeopathy Colleges Register</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Commission for Homoeopathy (NCH)</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>quality_status</t>
+          <t>S.No (NCH)</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F94" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F94" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
@@ -7851,54 +8779,54 @@
       </c>
       <c r="H94" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr">
         <is>
-          <t>PASS, WARNING, NEEDS REVIEW</t>
+          <t>Sequential serial number (1–299)</t>
         </is>
       </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
-          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+          <t>Gazetted institution serial number from the official NCH AY 2026-27 permission status document.</t>
         </is>
       </c>
       <c r="K94" s="4" t="inlineStr">
         <is>
-          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+          <t>100% sequential across all 25 pages with zero gaps.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NCH Homoeopathy Colleges Register</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Commission for Homoeopathy (NCH)</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>review_priority</t>
+          <t>Institution Name</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F95" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F95" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
@@ -7908,44 +8836,44 @@
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>Dr. Allu Ramalingaiah Government Homoeopathic Medical College</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>HIGH, MEDIUM, LOW</t>
+          <t>Official registered homoeopathic college title</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
         <is>
-          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+          <t>Standardized, deduplicated official name of the homoeopathic institution, parsed cleanly from the composite header address text.</t>
         </is>
       </c>
       <c r="K95" s="4" t="inlineStr">
         <is>
-          <t>Calculated from quality_status and missing data thresholds.</t>
+          <t>100% populated. No missing college names.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NCH Homoeopathy Colleges Register</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Commission for Homoeopathy (NCH)</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>canonical_state</t>
+          <t>Full Name &amp; Address</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -7953,9 +8881,9 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F96" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F96" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
@@ -7965,44 +8893,44 @@
       </c>
       <c r="H96" s="4" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Dr. Allu Ramalingaiah Govt. Homoeo Medical College, D.No. 26-1-11, V.L. Puram, Rajahmundry-533103, East Godavari Distt.</t>
         </is>
       </c>
       <c r="I96" s="4" t="inlineStr">
         <is>
-          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+          <t>Verbatim institution address and locality string</t>
         </is>
       </c>
       <c r="J96" s="4" t="inlineStr">
         <is>
-          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+          <t>Raw unparsed text string from NCH PDF containing college name, postal address, street, district, PIN code, and contact information.</t>
         </is>
       </c>
       <c r="K96" s="4" t="inlineStr">
         <is>
-          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+          <t>Primary source textual record for institutional entity verification.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NCH Homoeopathy Colleges Register</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Commission for Homoeopathy (NCH)</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>inferred_district</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -8010,9 +8938,9 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F97" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F97" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
@@ -8022,77 +8950,1160 @@
       </c>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>Ranga Reddy</t>
+          <t>arghmcrjy@gmail.com</t>
         </is>
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>Known Indian district name, or 'Not Specified'</t>
+          <t>Valid email address or empty</t>
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr">
         <is>
-          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+          <t>Administrative or institutional principal contact email address parsed from the composite address block using regex pattern matching.</t>
         </is>
       </c>
       <c r="K97" s="4" t="inlineStr">
         <is>
-          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+          <t>Extracted where present in official directory.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>Pincode</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="F98" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>533103</t>
+        </is>
+      </c>
+      <c r="I98" s="4" t="inlineStr">
+        <is>
+          <t>6-digit Indian PIN code</t>
+        </is>
+      </c>
+      <c r="J98" s="4" t="inlineStr">
+        <is>
+          <t>Six-digit postal index number extracted from the campus address block.</t>
+        </is>
+      </c>
+      <c r="K98" s="4" t="inlineStr">
+        <is>
+          <t>Extracted with boundary validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D99" s="9" t="inlineStr">
+        <is>
+          <t>State/UT</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F99" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>Standard 36 States/UTs</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr">
+        <is>
+          <t>State or Union Territory heading under which the homoeopathic college is officially registered by NCH.</t>
+        </is>
+      </c>
+      <c r="K99" s="4" t="inlineStr">
+        <is>
+          <t>Covers 26 States and UTs offering recognized homoeopathic medical education.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="inlineStr">
+        <is>
+          <t>NCH College Code</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F100" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>Yes (Where Assigned)</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="I100" s="4" t="inlineStr">
+        <is>
+          <t>Official MARBH/NCH numeric or alphanumeric college code</t>
+        </is>
+      </c>
+      <c r="J100" s="4" t="inlineStr">
+        <is>
+          <t>Statutory regulatory identifier assigned to the college by the Medical Assessment and Rating Board for Homoeopathy (MARBH).</t>
+        </is>
+      </c>
+      <c r="K100" s="4" t="inlineStr">
+        <is>
+          <t>Official regulatory ID. 9 newly applied colleges lack pre-assigned codes and use deterministic canonical keys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="inlineStr">
+        <is>
+          <t>Identifier Type</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F101" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>NCH_COLLEGE_CODE</t>
+        </is>
+      </c>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
+          <t>NCH_COLLEGE_CODE, NCH_DERIVED_KEY</t>
+        </is>
+      </c>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>Audit classification indicating whether the college possesses an official MARBH code or a synthetic deterministic surrogate identifier.</t>
+        </is>
+      </c>
+      <c r="K101" s="4" t="inlineStr">
+        <is>
+          <t>Provides transparency on regulatory ID presence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>Canonical Key</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F102" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>NCH_101</t>
+        </is>
+      </c>
+      <c r="I102" s="4" t="inlineStr">
+        <is>
+          <t>NCH_&lt;CODE&gt; or NCH_DERIVED_&lt;SNO&gt;</t>
+        </is>
+      </c>
+      <c r="J102" s="4" t="inlineStr">
+        <is>
+          <t>Normalized, immutable institutional key used for national multi-source cross-registry linking.</t>
+        </is>
+      </c>
+      <c r="K102" s="4" t="inlineStr">
+        <is>
+          <t>Ensures unique index representation in master census.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>Management Type</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F103" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>Govt.</t>
+        </is>
+      </c>
+      <c r="I103" s="4" t="inlineStr">
+        <is>
+          <t>Govt., Pvt. (Private), Trust, Society, Grant-in-aid</t>
+        </is>
+      </c>
+      <c r="J103" s="4" t="inlineStr">
+        <is>
+          <t>Institutional governance and ownership model (Government vs Private/Trust).</t>
+        </is>
+      </c>
+      <c r="K103" s="4" t="inlineStr">
+        <is>
+          <t>Normalized from raw 'Govt/Pvt' PDF column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>UG Seat Intake</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="F104" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H104" s="4" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="I104" s="4" t="inlineStr">
+        <is>
+          <t>Numeric seat capacity or 'Nil' / '-'</t>
+        </is>
+      </c>
+      <c r="J104" s="4" t="inlineStr">
+        <is>
+          <t>Undergraduate Bachelor of Homoeopathic Medicine and Surgery (BHMS) annual student admission intake capacity applied for or permitted.</t>
+        </is>
+      </c>
+      <c r="K104" s="4" t="inlineStr">
+        <is>
+          <t>Applicable for UG-granting institutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>UG Permission</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="F105" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="I105" s="4" t="inlineStr">
+        <is>
+          <t>Numeric permitted seats (including EWS quota) or '-'</t>
+        </is>
+      </c>
+      <c r="J105" s="4" t="inlineStr">
+        <is>
+          <t>Number of undergraduate BHMS seats officially approved and permitted by MARBH for the academic session 2026-27.</t>
+        </is>
+      </c>
+      <c r="K105" s="4" t="inlineStr">
+        <is>
+          <t>Zero or '-' indicates admission denial or withheld status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>PG Seat Intake</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="F106" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H106" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="I106" s="4" t="inlineStr">
+        <is>
+          <t>Numeric seat capacity or '-'</t>
+        </is>
+      </c>
+      <c r="J106" s="4" t="inlineStr">
+        <is>
+          <t>Postgraduate MD (Homoeopathy) student intake capacity applied for or recognized.</t>
+        </is>
+      </c>
+      <c r="K106" s="4" t="inlineStr">
+        <is>
+          <t>Applicable for PG specialty colleges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>PG Permission</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="F107" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="I107" s="4" t="inlineStr">
+        <is>
+          <t>Numeric permitted PG seats or '-'</t>
+        </is>
+      </c>
+      <c r="J107" s="4" t="inlineStr">
+        <is>
+          <t>Total postgraduate seats approved by MARBH across clinical and non-clinical homoeopathic disciplines for AY 2026-27.</t>
+        </is>
+      </c>
+      <c r="K107" s="4" t="inlineStr">
+        <is>
+          <t>Subject-wise allocations detailed in companion column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>MARBH Decision</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F108" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H108" s="4" t="inlineStr">
+        <is>
+          <t>Conditional Permission</t>
+        </is>
+      </c>
+      <c r="I108" s="4" t="inlineStr">
+        <is>
+          <t>Permission, Conditional Permission, Denial, Permission Withheld, Status Not Available</t>
+        </is>
+      </c>
+      <c r="J108" s="4" t="inlineStr">
+        <is>
+          <t>Official regulatory determination issued by the Medical Assessment and Rating Board for Homoeopathy regarding college inspection and compliance.</t>
+        </is>
+      </c>
+      <c r="K108" s="4" t="inlineStr">
+        <is>
+          <t>Key statutory quality indicator governing student admissions for 2026-27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="inlineStr">
+        <is>
+          <t>Overall Permission Status</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F109" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>Conditional Permission</t>
+        </is>
+      </c>
+      <c r="I109" s="4" t="inlineStr">
+        <is>
+          <t>Conditional Permission (93), Status Not Available (114), Permission (52), Denial (39), Permission Withheld (1)</t>
+        </is>
+      </c>
+      <c r="J109" s="4" t="inlineStr">
+        <is>
+          <t>Normalized categorical status representing the institution's operational approval standing.</t>
+        </is>
+      </c>
+      <c r="K109" s="4" t="inlineStr">
+        <is>
+          <t>Enables executive filtering and quality dashboard visualization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>Scheme</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F110" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H110" s="4" t="inlineStr">
+        <is>
+          <t>UG &amp; PG</t>
+        </is>
+      </c>
+      <c r="I110" s="4" t="inlineStr">
+        <is>
+          <t>UG, PG, UG &amp; PG</t>
+        </is>
+      </c>
+      <c r="J110" s="4" t="inlineStr">
+        <is>
+          <t>Educational program tier authorized at the institution (Undergraduate, Postgraduate, or Both).</t>
+        </is>
+      </c>
+      <c r="K110" s="4" t="inlineStr">
+        <is>
+          <t>Delineates institutional scope of medical training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="inlineStr">
+        <is>
+          <t>Academic Year</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F111" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H111" s="4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="I111" s="4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="J111" s="4" t="inlineStr">
+        <is>
+          <t>Academic cycle for which the statutory permission status and seat intake quota apply.</t>
+        </is>
+      </c>
+      <c r="K111" s="4" t="inlineStr">
+        <is>
+          <t>Current active AY under MARBH/NCH Gazette.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>NCH Homoeopathy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>National Commission for Homoeopathy (NCH)</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>URL (String)</t>
+        </is>
+      </c>
+      <c r="F112" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H112" s="4" t="inlineStr">
+        <is>
+          <t>https://nch.org.in/upload/Permission-Status%20as%20on%2003-08-2026.pdf</t>
+        </is>
+      </c>
+      <c r="I112" s="4" t="inlineStr">
+        <is>
+          <t>Valid HTTPS URL on official nch.org.in portal</t>
+        </is>
+      </c>
+      <c r="J112" s="4" t="inlineStr">
+        <is>
+          <t>Direct canonical link to the official regulatory PDF document published on the NCH portal.</t>
+        </is>
+      </c>
+      <c r="K112" s="4" t="inlineStr">
+        <is>
+          <t>Ensures complete data auditability and statutory lineage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B113" s="4" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C98" s="5" t="inlineStr">
+      <c r="C113" s="5" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D98" s="9" t="inlineStr">
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>quality_status</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F113" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H113" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I113" s="4" t="inlineStr">
+        <is>
+          <t>PASS, WARNING, NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="J113" s="4" t="inlineStr">
+        <is>
+          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+        </is>
+      </c>
+      <c r="K113" s="4" t="inlineStr">
+        <is>
+          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="inlineStr">
+        <is>
+          <t>review_priority</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F114" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H114" s="4" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I114" s="4" t="inlineStr">
+        <is>
+          <t>HIGH, MEDIUM, LOW</t>
+        </is>
+      </c>
+      <c r="J114" s="4" t="inlineStr">
+        <is>
+          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+        </is>
+      </c>
+      <c r="K114" s="4" t="inlineStr">
+        <is>
+          <t>Calculated from quality_status and missing data thresholds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>canonical_state</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F115" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H115" s="4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="I115" s="4" t="inlineStr">
+        <is>
+          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+        </is>
+      </c>
+      <c r="J115" s="4" t="inlineStr">
+        <is>
+          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+        </is>
+      </c>
+      <c r="K115" s="4" t="inlineStr">
+        <is>
+          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="inlineStr">
+        <is>
+          <t>inferred_district</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F116" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H116" s="4" t="inlineStr">
+        <is>
+          <t>Ranga Reddy</t>
+        </is>
+      </c>
+      <c r="I116" s="4" t="inlineStr">
+        <is>
+          <t>Known Indian district name, or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="J116" s="4" t="inlineStr">
+        <is>
+          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+        </is>
+      </c>
+      <c r="K116" s="4" t="inlineStr">
+        <is>
+          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
         <is>
           <t>_search_blob</t>
         </is>
       </c>
-      <c r="E98" s="5" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F98" s="12" t="inlineStr">
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F117" s="12" t="inlineStr">
         <is>
           <t>DASHBOARD-CALCULATED FIELD</t>
         </is>
       </c>
-      <c r="G98" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H98" s="4" t="inlineStr">
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H117" s="4" t="inlineStr">
         <is>
           <t>iiit hyderabad international institute of information technology gachibowli telangana 500032</t>
         </is>
       </c>
-      <c r="I98" s="4" t="inlineStr">
+      <c r="I117" s="4" t="inlineStr">
         <is>
           <t>Lowercase normalized concatenated search token string</t>
         </is>
       </c>
-      <c r="J98" s="4" t="inlineStr">
+      <c r="J117" s="4" t="inlineStr">
         <is>
           <t>Unified multi-attribute token string combining Name, State, District, Address, PIN, ID, University, and Locality Aliases for fast sub-millisecond global search.</t>
         </is>
       </c>
-      <c r="K98" s="4" t="inlineStr">
+      <c r="K117" s="4" t="inlineStr">
         <is>
           <t>Powers /api/search and in-table search across all 7,335 final list records.</t>
         </is>

</xml_diff>

<commit_message>
Complete BCI Law Colleges dataset (3,074 CLEs across 31 States/UTs), update Data Dictionary and roadmap
</commit_message>
<xml_diff>
--- a/DATA_DICTIONARY.xlsx
+++ b/DATA_DICTIONARY.xlsx
@@ -20,7 +20,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CISCE_Schools" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telangana_Census" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NCH_Homoeopathy" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Calculated" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCI_Law" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Calculated" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -531,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -539,7 +540,7 @@
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -1227,53 +1228,108 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Legal Education (LL.B / Integrated Law / LL.M)</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>3,074</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>31 / 36 (86%)</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>BCI_College_ID (e.g. S35U10C24)</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>Bar Council of India Statutory CLE Register (BCA0026X2518XJCSA38.pdf)</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>100% complete national census of recognized/approved Centres of Legal Education (CLEs) across India under Advocates Act, 1961.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Cross-Cutting Metadata &amp; Search</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>7,335 Final Records</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>10,708 Final Records</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>36 / 36 (100%)</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>N/A (Derived Attributes)</t>
         </is>
       </c>
-      <c r="I16" s="7" t="n">
+      <c r="I17" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>Pan-India Data Quality &amp; Deduplication Engine</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Standardized canonical state, inferred district, quality status, and search blobs.</t>
         </is>
@@ -3140,6 +3196,752 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DATA DICTIONARY: BCI NATIONAL LAW COLLEGES REGISTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Field / Column Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Field Classification</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Required?</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Example Value</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Allowed Values / Codebook</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Description / Meaning</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Methodological Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>1 to 3074</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Sequential institutional index in the pan-India census.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Generated during state-wise sorting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Institution Name</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Veeravalli College of Law</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Approved Centre of Legal Education name</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Official statutory name of the law college or university legal department.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Verified against BCI master roster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>One of 36 Canonical States &amp; UTs</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>State or Union Territory where the institution is physically located.</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Standardized to official census state names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>East Godavari</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>LGD Official 787 Districts</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Administrative district resolved against Local Government Directory master.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from location string and verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Rajahmundry</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>City / Town name</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Urban agglomeration or municipality of the campus.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Parsed from college place tokens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Veeravalli College of Law, Rajahmundry, Dist. East Godavari, Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Complete address string</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Full postal location and campus description.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Combines institution name, location, district, and state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>University / Affiliating University</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Adikavi Nannaya University, Rajamahendravaram</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Recognized UGC university name</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Statutory degree-awarding university to which the law college is affiliated.</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Matches BCI statutory affiliation orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Management Type</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Private / Trust</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Government, University Constituent / Dept, Government Aided, Private / Trust</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Institutional governance classification.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Inferred from ownership, statutory charters, and naming conventions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Approval Status</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Approved / Recognized</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Approved / Recognized, Prohibited from Admission, Closed / Discontinued</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Current regulatory standing under BCI Legal Education Rules.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Reflects latest inspection and compliance status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Programmes / Courses</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>3 year LLB Course (180); 5 year BA LLB Course (120)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Semicolon-separated course list with intake strength</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>All legal education degree courses authorized at this physical campus.</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Aggregated across all approved course entries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>BCI College ID</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>S02U01C01</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Official BCI online code (S..U..C..) or canonical census key (BCI_..)</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Official unique institutional code assigned by Bar Council of India.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Primary regulatory identifier for legal education institutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Approval Year / Academic Year</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Upto 2026-27</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Academic year string (e.g. Upto 2026-27)</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Validity period of statutory affiliation approval granted by BCI.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Indicates current inspection compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Year of Establishment</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>4-digit year</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Founding year of the law college.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Recorded in BCI historical inspection files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Regularised for AY 2023-24</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Free text notes from BCI Council</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Official comments and stipulations issued by the Legal Education Committee.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Provides compliance and regularization context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>URL (String)</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.barcouncilofindia.org/info/recognised-universities-colleges</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Valid HTTPS URL on official barcouncilofindia.org portal</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Canonical link to official BCI portal directory.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Ensures complete lineage to statutory source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Collection Date</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Date (ISO 8601)</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Date on which data was retrieved and verified from BCI.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Audit timestamp.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3424,13 +4226,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K117"/>
+  <dimension ref="A1:K133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="29" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
@@ -9827,32 +10629,32 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>BCI National Law Colleges Register</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>Bar Council of India (BCI)</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>quality_status</t>
+          <t>S.No</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F113" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F113" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G113" s="5" t="inlineStr">
@@ -9862,54 +10664,54 @@
       </c>
       <c r="H113" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>PASS, WARNING, NEEDS REVIEW</t>
+          <t>1 to 3074</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
         <is>
-          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+          <t>Sequential institutional index in the pan-India census.</t>
         </is>
       </c>
       <c r="K113" s="4" t="inlineStr">
         <is>
-          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+          <t>Generated during state-wise sorting.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>BCI National Law Colleges Register</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>Bar Council of India (BCI)</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D114" s="9" t="inlineStr">
         <is>
-          <t>review_priority</t>
+          <t>Institution Name</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F114" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F114" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G114" s="5" t="inlineStr">
@@ -9919,44 +10721,44 @@
       </c>
       <c r="H114" s="4" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>Veeravalli College of Law</t>
         </is>
       </c>
       <c r="I114" s="4" t="inlineStr">
         <is>
-          <t>HIGH, MEDIUM, LOW</t>
+          <t>Approved Centre of Legal Education name</t>
         </is>
       </c>
       <c r="J114" s="4" t="inlineStr">
         <is>
-          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+          <t>Official statutory name of the law college or university legal department.</t>
         </is>
       </c>
       <c r="K114" s="4" t="inlineStr">
         <is>
-          <t>Calculated from quality_status and missing data thresholds.</t>
+          <t>Verified against BCI master roster.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>BCI National Law Colleges Register</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>Bar Council of India (BCI)</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D115" s="9" t="inlineStr">
         <is>
-          <t>canonical_state</t>
+          <t>State</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
@@ -9964,9 +10766,9 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F115" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F115" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G115" s="5" t="inlineStr">
@@ -9981,39 +10783,39 @@
       </c>
       <c r="I115" s="4" t="inlineStr">
         <is>
-          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+          <t>One of 36 Canonical States &amp; UTs</t>
         </is>
       </c>
       <c r="J115" s="4" t="inlineStr">
         <is>
-          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+          <t>State or Union Territory where the institution is physically located.</t>
         </is>
       </c>
       <c r="K115" s="4" t="inlineStr">
         <is>
-          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+          <t>Standardized to official census state names.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>BCI National Law Colleges Register</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>Bar Council of India (BCI)</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr">
         <is>
-          <t>inferred_district</t>
+          <t>District</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
@@ -10021,89 +10823,1001 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F116" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F116" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
         </is>
       </c>
       <c r="G116" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H116" s="4" t="inlineStr">
         <is>
-          <t>Ranga Reddy</t>
+          <t>East Godavari</t>
         </is>
       </c>
       <c r="I116" s="4" t="inlineStr">
         <is>
-          <t>Known Indian district name, or 'Not Specified'</t>
+          <t>LGD Official 787 Districts</t>
         </is>
       </c>
       <c r="J116" s="4" t="inlineStr">
         <is>
-          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+          <t>Administrative district resolved against Local Government Directory master.</t>
         </is>
       </c>
       <c r="K116" s="4" t="inlineStr">
         <is>
-          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+          <t>Extracted from location string and verified.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F117" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>Rajahmundry</t>
+        </is>
+      </c>
+      <c r="I117" s="4" t="inlineStr">
+        <is>
+          <t>City / Town name</t>
+        </is>
+      </c>
+      <c r="J117" s="4" t="inlineStr">
+        <is>
+          <t>Urban agglomeration or municipality of the campus.</t>
+        </is>
+      </c>
+      <c r="K117" s="4" t="inlineStr">
+        <is>
+          <t>Parsed from college place tokens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F118" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G118" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H118" s="4" t="inlineStr">
+        <is>
+          <t>Veeravalli College of Law, Rajahmundry, Dist. East Godavari, Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="I118" s="4" t="inlineStr">
+        <is>
+          <t>Complete address string</t>
+        </is>
+      </c>
+      <c r="J118" s="4" t="inlineStr">
+        <is>
+          <t>Full postal location and campus description.</t>
+        </is>
+      </c>
+      <c r="K118" s="4" t="inlineStr">
+        <is>
+          <t>Combines institution name, location, district, and state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>University / Affiliating University</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F119" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>Adikavi Nannaya University, Rajamahendravaram</t>
+        </is>
+      </c>
+      <c r="I119" s="4" t="inlineStr">
+        <is>
+          <t>Recognized UGC university name</t>
+        </is>
+      </c>
+      <c r="J119" s="4" t="inlineStr">
+        <is>
+          <t>Statutory degree-awarding university to which the law college is affiliated.</t>
+        </is>
+      </c>
+      <c r="K119" s="4" t="inlineStr">
+        <is>
+          <t>Matches BCI statutory affiliation orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>Management Type</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F120" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G120" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H120" s="4" t="inlineStr">
+        <is>
+          <t>Private / Trust</t>
+        </is>
+      </c>
+      <c r="I120" s="4" t="inlineStr">
+        <is>
+          <t>Government, University Constituent / Dept, Government Aided, Private / Trust</t>
+        </is>
+      </c>
+      <c r="J120" s="4" t="inlineStr">
+        <is>
+          <t>Institutional governance classification.</t>
+        </is>
+      </c>
+      <c r="K120" s="4" t="inlineStr">
+        <is>
+          <t>Inferred from ownership, statutory charters, and naming conventions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>Approval Status</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F121" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>Approved / Recognized</t>
+        </is>
+      </c>
+      <c r="I121" s="4" t="inlineStr">
+        <is>
+          <t>Approved / Recognized, Prohibited from Admission, Closed / Discontinued</t>
+        </is>
+      </c>
+      <c r="J121" s="4" t="inlineStr">
+        <is>
+          <t>Current regulatory standing under BCI Legal Education Rules.</t>
+        </is>
+      </c>
+      <c r="K121" s="4" t="inlineStr">
+        <is>
+          <t>Reflects latest inspection and compliance status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D122" s="9" t="inlineStr">
+        <is>
+          <t>Programmes / Courses</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F122" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H122" s="4" t="inlineStr">
+        <is>
+          <t>3 year LLB Course (180); 5 year BA LLB Course (120)</t>
+        </is>
+      </c>
+      <c r="I122" s="4" t="inlineStr">
+        <is>
+          <t>Semicolon-separated course list with intake strength</t>
+        </is>
+      </c>
+      <c r="J122" s="4" t="inlineStr">
+        <is>
+          <t>All legal education degree courses authorized at this physical campus.</t>
+        </is>
+      </c>
+      <c r="K122" s="4" t="inlineStr">
+        <is>
+          <t>Aggregated across all approved course entries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>BCI College ID</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F123" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>S02U01C01</t>
+        </is>
+      </c>
+      <c r="I123" s="4" t="inlineStr">
+        <is>
+          <t>Official BCI online code (S..U..C..) or canonical census key (BCI_..)</t>
+        </is>
+      </c>
+      <c r="J123" s="4" t="inlineStr">
+        <is>
+          <t>Official unique institutional code assigned by Bar Council of India.</t>
+        </is>
+      </c>
+      <c r="K123" s="4" t="inlineStr">
+        <is>
+          <t>Primary regulatory identifier for legal education institutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>Approval Year / Academic Year</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F124" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G124" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H124" s="4" t="inlineStr">
+        <is>
+          <t>Upto 2026-27</t>
+        </is>
+      </c>
+      <c r="I124" s="4" t="inlineStr">
+        <is>
+          <t>Academic year string (e.g. Upto 2026-27)</t>
+        </is>
+      </c>
+      <c r="J124" s="4" t="inlineStr">
+        <is>
+          <t>Validity period of statutory affiliation approval granted by BCI.</t>
+        </is>
+      </c>
+      <c r="K124" s="4" t="inlineStr">
+        <is>
+          <t>Indicates current inspection compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>Year of Establishment</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F125" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="I125" s="4" t="inlineStr">
+        <is>
+          <t>4-digit year</t>
+        </is>
+      </c>
+      <c r="J125" s="4" t="inlineStr">
+        <is>
+          <t>Founding year of the law college.</t>
+        </is>
+      </c>
+      <c r="K125" s="4" t="inlineStr">
+        <is>
+          <t>Recorded in BCI historical inspection files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F126" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G126" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t>Regularised for AY 2023-24</t>
+        </is>
+      </c>
+      <c r="I126" s="4" t="inlineStr">
+        <is>
+          <t>Free text notes from BCI Council</t>
+        </is>
+      </c>
+      <c r="J126" s="4" t="inlineStr">
+        <is>
+          <t>Official comments and stipulations issued by the Legal Education Committee.</t>
+        </is>
+      </c>
+      <c r="K126" s="4" t="inlineStr">
+        <is>
+          <t>Provides compliance and regularization context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>URL (String)</t>
+        </is>
+      </c>
+      <c r="F127" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G127" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t>https://www.barcouncilofindia.org/info/recognised-universities-colleges</t>
+        </is>
+      </c>
+      <c r="I127" s="4" t="inlineStr">
+        <is>
+          <t>Valid HTTPS URL on official barcouncilofindia.org portal</t>
+        </is>
+      </c>
+      <c r="J127" s="4" t="inlineStr">
+        <is>
+          <t>Canonical link to official BCI portal directory.</t>
+        </is>
+      </c>
+      <c r="K127" s="4" t="inlineStr">
+        <is>
+          <t>Ensures complete lineage to statutory source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>BCI National Law Colleges Register</t>
+        </is>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>Bar Council of India (BCI)</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>Collection Date</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>Date (ISO 8601)</t>
+        </is>
+      </c>
+      <c r="F128" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G128" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+      <c r="J128" s="4" t="inlineStr">
+        <is>
+          <t>Date on which data was retrieved and verified from BCI.</t>
+        </is>
+      </c>
+      <c r="K128" s="4" t="inlineStr">
+        <is>
+          <t>Audit timestamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B117" s="4" t="inlineStr">
+      <c r="B129" s="4" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C117" s="5" t="inlineStr">
+      <c r="C129" s="5" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D117" s="9" t="inlineStr">
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>quality_status</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F129" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G129" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I129" s="4" t="inlineStr">
+        <is>
+          <t>PASS, WARNING, NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="J129" s="4" t="inlineStr">
+        <is>
+          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+        </is>
+      </c>
+      <c r="K129" s="4" t="inlineStr">
+        <is>
+          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>review_priority</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F130" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G130" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H130" s="4" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I130" s="4" t="inlineStr">
+        <is>
+          <t>HIGH, MEDIUM, LOW</t>
+        </is>
+      </c>
+      <c r="J130" s="4" t="inlineStr">
+        <is>
+          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+        </is>
+      </c>
+      <c r="K130" s="4" t="inlineStr">
+        <is>
+          <t>Calculated from quality_status and missing data thresholds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>canonical_state</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F131" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G131" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H131" s="4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="I131" s="4" t="inlineStr">
+        <is>
+          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+        </is>
+      </c>
+      <c r="J131" s="4" t="inlineStr">
+        <is>
+          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+        </is>
+      </c>
+      <c r="K131" s="4" t="inlineStr">
+        <is>
+          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
+        <is>
+          <t>inferred_district</t>
+        </is>
+      </c>
+      <c r="E132" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F132" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G132" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H132" s="4" t="inlineStr">
+        <is>
+          <t>Ranga Reddy</t>
+        </is>
+      </c>
+      <c r="I132" s="4" t="inlineStr">
+        <is>
+          <t>Known Indian district name, or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="J132" s="4" t="inlineStr">
+        <is>
+          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+        </is>
+      </c>
+      <c r="K132" s="4" t="inlineStr">
+        <is>
+          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
         <is>
           <t>_search_blob</t>
         </is>
       </c>
-      <c r="E117" s="5" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F117" s="12" t="inlineStr">
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F133" s="12" t="inlineStr">
         <is>
           <t>DASHBOARD-CALCULATED FIELD</t>
         </is>
       </c>
-      <c r="G117" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H117" s="4" t="inlineStr">
+      <c r="G133" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H133" s="4" t="inlineStr">
         <is>
           <t>iiit hyderabad international institute of information technology gachibowli telangana 500032</t>
         </is>
       </c>
-      <c r="I117" s="4" t="inlineStr">
+      <c r="I133" s="4" t="inlineStr">
         <is>
           <t>Lowercase normalized concatenated search token string</t>
         </is>
       </c>
-      <c r="J117" s="4" t="inlineStr">
+      <c r="J133" s="4" t="inlineStr">
         <is>
           <t>Unified multi-attribute token string combining Name, State, District, Address, PIN, ID, University, and Locality Aliases for fast sub-millisecond global search.</t>
         </is>
       </c>
-      <c r="K117" s="4" t="inlineStr">
+      <c r="K133" s="4" t="inlineStr">
         <is>
           <t>Powers /api/search and in-table search across all 7,335 final list records.</t>
         </is>

</xml_diff>

<commit_message>
Complete PCI Pharmacy Colleges dataset (6,664 institutions across 32 States/UTs), update Data Dictionary, roadmap and dashboard
</commit_message>
<xml_diff>
--- a/DATA_DICTIONARY.xlsx
+++ b/DATA_DICTIONARY.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1283,53 +1283,108 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Education (D.Pharm / B.Pharm / M.Pharm / Pharm.D)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>6,664</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>32 / 36 (89%)</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>PCI_College_ID (e.g. PCI-1, PCI-6)</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India Statutory Register (16,033 stream filings)</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>100% complete national census of recognized/approved pharmacy colleges across India under Pharmacy Act, 1948.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Cross-Cutting Metadata &amp; Search</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>10,708 Final Records</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>36 / 36 (100%)</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>N/A (Derived Attributes)</t>
         </is>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="I18" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>Pan-India Data Quality &amp; Deduplication Engine</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>Standardized canonical state, inferred district, quality status, and search blobs.</t>
         </is>
@@ -4226,7 +4281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K133"/>
+  <dimension ref="A1:K149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -11541,32 +11596,32 @@
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>PCI National Pharmacy Colleges Register</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>Pharmacy Council of India (PCI)</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D129" s="9" t="inlineStr">
         <is>
-          <t>quality_status</t>
+          <t>S.No</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F129" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F129" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
         </is>
       </c>
       <c r="G129" s="5" t="inlineStr">
@@ -11576,54 +11631,54 @@
       </c>
       <c r="H129" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I129" s="4" t="inlineStr">
         <is>
-          <t>PASS, WARNING, NEEDS REVIEW</t>
+          <t>Sequential positive integers (1 to 6,664)</t>
         </is>
       </c>
       <c r="J129" s="4" t="inlineStr">
         <is>
-          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+          <t>Sequential identifier assigned during reconciliation of the national physical pharmacy college register.</t>
         </is>
       </c>
       <c r="K129" s="4" t="inlineStr">
         <is>
-          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+          <t>Provides fixed row reference across the deduplicated roster.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>PCI National Pharmacy Colleges Register</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>Pharmacy Council of India (PCI)</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D130" s="9" t="inlineStr">
         <is>
-          <t>review_priority</t>
+          <t>Institution Name</t>
         </is>
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F130" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F130" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G130" s="5" t="inlineStr">
@@ -11633,44 +11688,44 @@
       </c>
       <c r="H130" s="4" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>Advance Institute Of Biotech And Paramedical Sciences</t>
         </is>
       </c>
       <c r="I130" s="4" t="inlineStr">
         <is>
-          <t>HIGH, MEDIUM, LOW</t>
+          <t>Official statutory name of the pharmacy institution</t>
         </is>
       </c>
       <c r="J130" s="4" t="inlineStr">
         <is>
-          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+          <t>Cleaned legal name of the pharmacy institution/college recognized under the Pharmacy Act, 1948.</t>
         </is>
       </c>
       <c r="K130" s="4" t="inlineStr">
         <is>
-          <t>Calculated from quality_status and missing data thresholds.</t>
+          <t>Consolidated across course streams; captures the primary physical institution entity.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>PCI National Pharmacy Colleges Register</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>Pharmacy Council of India (PCI)</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D131" s="9" t="inlineStr">
         <is>
-          <t>canonical_state</t>
+          <t>State</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
@@ -11678,9 +11733,9 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F131" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F131" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G131" s="5" t="inlineStr">
@@ -11690,44 +11745,44 @@
       </c>
       <c r="H131" s="4" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Uttar Pradesh</t>
         </is>
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+          <t>One of 36 Canonical Indian States or Union Territories</t>
         </is>
       </c>
       <c r="J131" s="4" t="inlineStr">
         <is>
-          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+          <t>State or Union Territory in which the pharmacy college campus is physically located.</t>
         </is>
       </c>
       <c r="K131" s="4" t="inlineStr">
         <is>
-          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+          <t>Standardized to canonical spelling across all 32 covered States/UTs.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>PCI National Pharmacy Colleges Register</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>Pharmacy Council of India (PCI)</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D132" s="9" t="inlineStr">
         <is>
-          <t>inferred_district</t>
+          <t>District</t>
         </is>
       </c>
       <c r="E132" s="5" t="inlineStr">
@@ -11735,9 +11790,9 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F132" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F132" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
         </is>
       </c>
       <c r="G132" s="5" t="inlineStr">
@@ -11747,77 +11802,989 @@
       </c>
       <c r="H132" s="4" t="inlineStr">
         <is>
-          <t>Ranga Reddy</t>
+          <t>Lucknow</t>
         </is>
       </c>
       <c r="I132" s="4" t="inlineStr">
         <is>
-          <t>Known Indian district name, or 'Not Specified'</t>
+          <t>Recognized Indian district name, or 'Not Specified'</t>
         </is>
       </c>
       <c r="J132" s="4" t="inlineStr">
         <is>
-          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+          <t>District administrative boundary extracted by cross-referencing state district masters and location tokens.</t>
         </is>
       </c>
       <c r="K132" s="4" t="inlineStr">
         <is>
-          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+          <t>89.6% district resolution achieved across 6,664 physical institutions.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F133" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G133" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H133" s="4" t="inlineStr">
+        <is>
+          <t>Lucknow</t>
+        </is>
+      </c>
+      <c r="I133" s="4" t="inlineStr">
+        <is>
+          <t>Town, city, or municipal locality</t>
+        </is>
+      </c>
+      <c r="J133" s="4" t="inlineStr">
+        <is>
+          <t>City or urban agglomeration serving the physical pharmacy college campus.</t>
+        </is>
+      </c>
+      <c r="K133" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from institutional address and district tokens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D134" s="9" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E134" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F134" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G134" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H134" s="4" t="inlineStr">
+        <is>
+          <t>Advance Institute Of Biotech And Paramedical Sciences Kanpur Road Lucknow</t>
+        </is>
+      </c>
+      <c r="I134" s="4" t="inlineStr">
+        <is>
+          <t>Full street/campus address string</t>
+        </is>
+      </c>
+      <c r="J134" s="4" t="inlineStr">
+        <is>
+          <t>Complete physical address including road, village, mandal, and district location tokens.</t>
+        </is>
+      </c>
+      <c r="K134" s="4" t="inlineStr">
+        <is>
+          <t>Preserves full campus geographical provenance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D135" s="9" t="inlineStr">
+        <is>
+          <t>University / Affiliating University</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F135" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G135" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H135" s="4" t="inlineStr">
+        <is>
+          <t>Dr. A.P.J. Abdul Kalam Technical University</t>
+        </is>
+      </c>
+      <c r="I135" s="4" t="inlineStr">
+        <is>
+          <t>Recognized university or state examining board</t>
+        </is>
+      </c>
+      <c r="J135" s="4" t="inlineStr">
+        <is>
+          <t>Statutory Examining Authority or University to which the pharmacy college is affiliated.</t>
+        </is>
+      </c>
+      <c r="K135" s="4" t="inlineStr">
+        <is>
+          <t>Cleaned from examiningauthority_name; captures both degree-granting universities and state technical boards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D136" s="9" t="inlineStr">
+        <is>
+          <t>Management Type</t>
+        </is>
+      </c>
+      <c r="E136" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F136" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G136" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H136" s="4" t="inlineStr">
+        <is>
+          <t>Private / Self-Financed</t>
+        </is>
+      </c>
+      <c r="I136" s="4" t="inlineStr">
+        <is>
+          <t>Government / University Constituent, Private / Self-Financed</t>
+        </is>
+      </c>
+      <c r="J136" s="4" t="inlineStr">
+        <is>
+          <t>Administrative ownership category inferred from institution and university designations.</t>
+        </is>
+      </c>
+      <c r="K136" s="4" t="inlineStr">
+        <is>
+          <t>Classified based on statutory ownership indicators.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D137" s="9" t="inlineStr">
+        <is>
+          <t>Approval Status</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F137" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G137" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H137" s="4" t="inlineStr">
+        <is>
+          <t>Approved u/s 12</t>
+        </is>
+      </c>
+      <c r="I137" s="4" t="inlineStr">
+        <is>
+          <t>Approved u/s 12, Approved for Conduct of Course, Approved u/s 12 &amp; Conduct of Course, Approved</t>
+        </is>
+      </c>
+      <c r="J137" s="4" t="inlineStr">
+        <is>
+          <t>Statutory regulatory approval status under Section 12 or conduct provisions of the Pharmacy Act, 1948.</t>
+        </is>
+      </c>
+      <c r="K137" s="4" t="inlineStr">
+        <is>
+          <t>Indicates whether qualifying examinations are approved for registration as a registered pharmacist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D138" s="9" t="inlineStr">
+        <is>
+          <t>Programmes / Courses</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F138" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G138" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H138" s="4" t="inlineStr">
+        <is>
+          <t>B.Pharm, D.Pharm, M.Pharm (Pharmaceutics)</t>
+        </is>
+      </c>
+      <c r="I138" s="4" t="inlineStr">
+        <is>
+          <t>Comma-separated pharmacy qualifications: D.Pharm, B.Pharm, M.Pharm, Pharm.D, Pharm.D (PB), Bridge Course</t>
+        </is>
+      </c>
+      <c r="J138" s="4" t="inlineStr">
+        <is>
+          <t>Consolidated list of all PCI-approved programmes offered at this physical campus.</t>
+        </is>
+      </c>
+      <c r="K138" s="4" t="inlineStr">
+        <is>
+          <t>Unified from 16,033 course-stream filings into a single physical college row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D139" s="9" t="inlineStr">
+        <is>
+          <t>PCI College ID</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>String (Identifier)</t>
+        </is>
+      </c>
+      <c r="F139" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H139" s="4" t="inlineStr">
+        <is>
+          <t>PCI-1</t>
+        </is>
+      </c>
+      <c r="I139" s="4" t="inlineStr">
+        <is>
+          <t>Official PCI Code pattern: PCI-\d+</t>
+        </is>
+      </c>
+      <c r="J139" s="4" t="inlineStr">
+        <is>
+          <t>Official unique regulatory institution code assigned by Pharmacy Council of India.</t>
+        </is>
+      </c>
+      <c r="K139" s="4" t="inlineStr">
+        <is>
+          <t>100% complete across all 6,664 institutions; serves as the primary canonical regulatory key.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D140" s="9" t="inlineStr">
+        <is>
+          <t>Approval Year / Academic Year</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F140" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G140" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H140" s="4" t="inlineStr">
+        <is>
+          <t>2026-2027</t>
+        </is>
+      </c>
+      <c r="I140" s="4" t="inlineStr">
+        <is>
+          <t>Academic year span (e.g. 2026-2027, 2025-2026) or 'Current Approval'</t>
+        </is>
+      </c>
+      <c r="J140" s="4" t="inlineStr">
+        <is>
+          <t>Academic session up to which PCI approval has been extended or granted.</t>
+        </is>
+      </c>
+      <c r="K140" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official Central Council / Executive Committee decision orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D141" s="9" t="inlineStr">
+        <is>
+          <t>Intake / Seats</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F141" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G141" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H141" s="4" t="inlineStr">
+        <is>
+          <t>Total: 160 (B.Pharm: 100, D.Pharm: 60)</t>
+        </is>
+      </c>
+      <c r="I141" s="4" t="inlineStr">
+        <is>
+          <t>Approved annual admissions count per course or council norms</t>
+        </is>
+      </c>
+      <c r="J141" s="4" t="inlineStr">
+        <is>
+          <t>Total approved student intake capacity across all active pharmacy programmes.</t>
+        </is>
+      </c>
+      <c r="K141" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from formal Council decision notifications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D142" s="9" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F142" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G142" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H142" s="4" t="inlineStr">
+        <is>
+          <t>Approved across 2 regulatory stream decision(s). Aadhaar Enabled Biometric Attendance System (AEBAS) implementation mandated.</t>
+        </is>
+      </c>
+      <c r="I142" s="4" t="inlineStr">
+        <is>
+          <t>Stream decision counts and regulatory directives</t>
+        </is>
+      </c>
+      <c r="J142" s="4" t="inlineStr">
+        <is>
+          <t>Council directives and multi-stream consolidation metadata.</t>
+        </is>
+      </c>
+      <c r="K142" s="4" t="inlineStr">
+        <is>
+          <t>Captures AEBAS compliance requirements and decision stream linkages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D143" s="9" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>URL (String)</t>
+        </is>
+      </c>
+      <c r="F143" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H143" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pci.gov.in/</t>
+        </is>
+      </c>
+      <c r="I143" s="4" t="inlineStr">
+        <is>
+          <t>Valid HTTPS URL on official pci.gov.in portal</t>
+        </is>
+      </c>
+      <c r="J143" s="4" t="inlineStr">
+        <is>
+          <t>Canonical link to official PCI approved institutions register.</t>
+        </is>
+      </c>
+      <c r="K143" s="4" t="inlineStr">
+        <is>
+          <t>Ensures complete statutory lineage to Pharmacy Council of India.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="4" t="inlineStr">
+        <is>
+          <t>PCI National Pharmacy Colleges Register</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>Pharmacy Council of India (PCI)</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D144" s="9" t="inlineStr">
+        <is>
+          <t>Collection Date</t>
+        </is>
+      </c>
+      <c r="E144" s="5" t="inlineStr">
+        <is>
+          <t>Date (ISO 8601)</t>
+        </is>
+      </c>
+      <c r="F144" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G144" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H144" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I144" s="4" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+      <c r="J144" s="4" t="inlineStr">
+        <is>
+          <t>Date on which data was retrieved and verified from PCI official portal.</t>
+        </is>
+      </c>
+      <c r="K144" s="4" t="inlineStr">
+        <is>
+          <t>Audit timestamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B133" s="4" t="inlineStr">
+      <c r="B145" s="4" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C133" s="5" t="inlineStr">
+      <c r="C145" s="5" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D133" s="9" t="inlineStr">
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>quality_status</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F145" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G145" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H145" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I145" s="4" t="inlineStr">
+        <is>
+          <t>PASS, WARNING, NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="J145" s="4" t="inlineStr">
+        <is>
+          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+        </is>
+      </c>
+      <c r="K145" s="4" t="inlineStr">
+        <is>
+          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D146" s="9" t="inlineStr">
+        <is>
+          <t>review_priority</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F146" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G146" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H146" s="4" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I146" s="4" t="inlineStr">
+        <is>
+          <t>HIGH, MEDIUM, LOW</t>
+        </is>
+      </c>
+      <c r="J146" s="4" t="inlineStr">
+        <is>
+          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+        </is>
+      </c>
+      <c r="K146" s="4" t="inlineStr">
+        <is>
+          <t>Calculated from quality_status and missing data thresholds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D147" s="9" t="inlineStr">
+        <is>
+          <t>canonical_state</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F147" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G147" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H147" s="4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="I147" s="4" t="inlineStr">
+        <is>
+          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+        </is>
+      </c>
+      <c r="J147" s="4" t="inlineStr">
+        <is>
+          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+        </is>
+      </c>
+      <c r="K147" s="4" t="inlineStr">
+        <is>
+          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D148" s="9" t="inlineStr">
+        <is>
+          <t>inferred_district</t>
+        </is>
+      </c>
+      <c r="E148" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F148" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G148" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H148" s="4" t="inlineStr">
+        <is>
+          <t>Ranga Reddy</t>
+        </is>
+      </c>
+      <c r="I148" s="4" t="inlineStr">
+        <is>
+          <t>Known Indian district name, or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="J148" s="4" t="inlineStr">
+        <is>
+          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+        </is>
+      </c>
+      <c r="K148" s="4" t="inlineStr">
+        <is>
+          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
         <is>
           <t>_search_blob</t>
         </is>
       </c>
-      <c r="E133" s="5" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F133" s="12" t="inlineStr">
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F149" s="12" t="inlineStr">
         <is>
           <t>DASHBOARD-CALCULATED FIELD</t>
         </is>
       </c>
-      <c r="G133" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H133" s="4" t="inlineStr">
+      <c r="G149" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H149" s="4" t="inlineStr">
         <is>
           <t>iiit hyderabad international institute of information technology gachibowli telangana 500032</t>
         </is>
       </c>
-      <c r="I133" s="4" t="inlineStr">
+      <c r="I149" s="4" t="inlineStr">
         <is>
           <t>Lowercase normalized concatenated search token string</t>
         </is>
       </c>
-      <c r="J133" s="4" t="inlineStr">
+      <c r="J149" s="4" t="inlineStr">
         <is>
           <t>Unified multi-attribute token string combining Name, State, District, Address, PIN, ID, University, and Locality Aliases for fast sub-millisecond global search.</t>
         </is>
       </c>
-      <c r="K133" s="4" t="inlineStr">
+      <c r="K149" s="4" t="inlineStr">
         <is>
           <t>Powers /api/search and in-table search across all 7,335 final list records.</t>
         </is>

</xml_diff>

<commit_message>
Add complete NCISM Ayurveda and Unani dataset
</commit_message>
<xml_diff>
--- a/DATA_DICTIONARY.xlsx
+++ b/DATA_DICTIONARY.xlsx
@@ -973,17 +973,17 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>650</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>12 / 36 (33%)</t>
+          <t>25 / 36 (69%)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -996,12 +996,12 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>NCISM AY 2025-26 Rating Roster</t>
+          <t>NCISM AY 2025-26 National Registries &amp; Permission Lists</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Rating roster of approved ISM colleges eligible for rating in AY 2025-26.</t>
+          <t>Full national universe (593 Ayurveda + 57 Unani = 650 physical institutions) from official NCISM registries enriched with AY 2025-26 permission circulars.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add official NDC dental colleges dataset
</commit_message>
<xml_diff>
--- a/DATA_DICTIONARY.xlsx
+++ b/DATA_DICTIONARY.xlsx
@@ -21,7 +21,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telangana_Census" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NCH_Homoeopathy" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCI_Law" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Calculated" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDC_Dental" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Calculated" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -532,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1338,53 +1339,108 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Dental Education (BDS / MDS / PG Diploma / DH / DM)</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>28 / 36 (78%)</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Official ID (e.g. 409, 3)</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>National Dental Commission Official College Search &amp; Portal Roster</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>100% complete national census of recognized/approved dental institutions across India under National Dental Commission Act, 2023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Cross-Cutting Metadata &amp; Search</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>10,708 Final Records</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>36 / 36 (100%)</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>N/A (Derived Attributes)</t>
         </is>
       </c>
-      <c r="I18" s="7" t="n">
+      <c r="I19" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>Pan-India Data Quality &amp; Deduplication Engine</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Standardized canonical state, inferred district, quality status, and search blobs.</t>
         </is>
@@ -3997,6 +4053,1298 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DATA DICTIONARY: NDC NATIONAL DENTAL COLLEGES REGISTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Field / Column Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Field Classification</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Required?</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Example Value</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Allowed Values / Codebook</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Description / Meaning</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Methodological Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>S.No.</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Sequential positive integers (1 to 330)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Sequential institutional index for enumeration in the Pan-India census roster.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Generated during census deduplication and synthesis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Official ID</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>409</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Unique numeric string portal ID assigned by NDC/DCI</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Authoritative institutional identifier assigned by the National Dental Commission / Dental Council of India portal.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Exposed in the College Search portal via SearchCollegeDetails.aspx?Id={id}. 100% unique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>College Name</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Anil Neerukonda Institute of Dental Sciences, Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Official registered dental institution title</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Full statutory name of the recognized dental college or institute.</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Extracted verbatim from the official College Search grid and detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Canonical Indian State or Union Territory name (28 States/UTs)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>State or Union Territory where the physical dental college campus is situated.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Harmonized to the national census canonical 36 States/UTs reference catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>District / City</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>District or municipality name, or 'PASS — SOURCE LIMITATION'</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Official city or district location of the dental college campus.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official detail page. Where absent in portal, marked 'PASS — SOURCE LIMITATION'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>PIN Code</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>531162</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>6-digit postal index number, or 'PASS — SOURCE LIMITATION'</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Postal index number of the dental college campus.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official college detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Establishment Year</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>2013-14</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Academic session or 4-digit calendar year (e.g. 1999-00, 2013-14)</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Academic year in which the dental college was officially established and permitted.</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Verified against official NDC College Search registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Institution Type</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>'Govt.', 'Private', 'Society', 'Trust', 'Autonomous'</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Regulatory ownership and operational classification of the dental institution.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Captured directly from official DCI search table and detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Management / Admin Authority</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Society</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>'Society', 'Trust', 'Government', 'Autonomous', 'PASS — SOURCE LIMITATION'</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Administrative authority, society, or trust running the dental institution.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official institution detail record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Affiliated University</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Dr. N T R University of Health Sciences, Vijayawada</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Name of affiliating health university, deemed university, or central institute</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Statutory health sciences or general university to which the dental college is affiliated.</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official DCI affiliation schedule table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Attached Hospital</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Anil Neerukonda Hospital</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Name of attached dental/general hospital or medical college</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Teaching or general hospital attached to the dental college for clinical training.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Mandatory statutory requirement under NDC regulations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Sangivalasa, visakhapatnam</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Campus address lines or 'PASS — SOURCE LIMITATION'</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Full street and campus location address lines.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Consolidated from Line 1 and Line 2 of official detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>BDS Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 100 seats</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats', 'Not Offered / None'</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Undergraduate Bachelor of Dental Surgery (BDS) offering status and permitted intake capacity.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Synthesized from course-level records for AY 2026-27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>BDS Seats</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer (0, 40, 50, 60, 100)</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Sanctioned annual undergraduate BDS student intake capacity.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official College Search permitted seats table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>MDS Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 40 seats (9 specialities)</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats ({M} specialities)', 'Not Offered / None'</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Postgraduate Master of Dental Surgery (MDS) status, total seats, and speciality diversity.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Aggregated from individual postgraduate speciality rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>MDS Seats</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer sum of all MDS speciality seats</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Aggregate annual postgraduate MDS student intake capacity across all specialities.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Summed across all official MDS speciality allocations for AY 2026-27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>PG Diploma Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 3 seats (1 specialities)</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats ({M} specialities)', 'Not Offered / None'</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Postgraduate Diploma course offering status and permitted intake capacity.</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from PG Diploma entries in official College Search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>PG Diploma Seats</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer (0, 1, 2, 3)</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Total sanctioned PG Diploma seats at the institution.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Summed across all PG Diploma allocations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>DH Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 20 seats (Recognised)</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats (Recognised)', 'Not Offered / Not Listed'</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Dental Hygienist (DH) diploma course recognition status and intake.</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Matched from official NDC/DCI DH statutory schedule (DH.pdf).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>DH Seats</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer (e.g. 0, 10, 20)</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Sanctioned Dental Hygienist course capacity.</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>0 if not recognized/approved to run Dental Hygienists course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>DM Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 20 seats (Recognized)</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats (Recognized)', 'Not Offered / Not Listed'</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Dental Mechanic (DM) diploma course recognition status and intake.</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Matched from official NDC/DCI DM statutory schedule (DM.pdf).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>DM Seats</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer (e.g. 0, 10, 20)</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Sanctioned Dental Mechanic course capacity.</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>0 if not recognized/approved to run Dental Mechanics course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Total Dental Intake Capacity</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Sum of BDS, MDS, PG Diploma, DH, and DM seats</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Total aggregate annual dental education student intake across all programs at the campus.</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Calculated field: BDS Seats + MDS Seats + PG Diploma Seats + DH Seats + DM Seats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Current Regulatory Status</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Recognised / Permitted</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>'Recognised / Permitted', 'Recognition Withdrawn', 'Admissions Stopped', 'Permission Disapproved', 'Permitted (Seats Reduced / Surrendered)', 'Permitted (Court Order / Sub-Judice)', 'Recognised / Permitted (Seats Revised)', 'Conditional / Regulatory Remark Noted'</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Harmonized regulatory approval and operational status under the NDC Act, 2023.</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Synthesized directly from official portal remarks without dropping any restricted institutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Regulatory Remarks</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>No adverse remarks on record</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Full verbatim regulatory note, or 'No adverse remarks on record'</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Verbatim statutory remarks, court orders, seat reduction directives, or withdrawal notices.</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Captured directly from the official portal's Remark column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Official Detail URL</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>https://dciindia.gov.in/SearchCollegeDetails.aspx?Id=409</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Official detail page URL on dciindia.gov.in</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Direct clickable link to the official college profile on the NDC/DCI portal.</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Preserves audit trail and public provenance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>https://dciindia.gov.in/CollegeSearch.aspx</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>https://dciindia.gov.in/CollegeSearch.aspx</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Authoritative primary source URL from which the national institutional data was harvested.</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Census primary source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Academic Year</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>'2026-27'</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Official regulatory academic session to which the permission and seat matrix applies.</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Standardized to official NDC session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Collection Date</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>ISO 8601 Date (YYYY-MM-DD)</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Date when the official NDC national college dataset was extracted.</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Timestamp of census compilation.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4281,7 +5629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K149"/>
+  <dimension ref="A1:K178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -12508,32 +13856,32 @@
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NDC National Dental Colleges Register</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D145" s="9" t="inlineStr">
         <is>
-          <t>quality_status</t>
+          <t>S.No.</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F145" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F145" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
         </is>
       </c>
       <c r="G145" s="5" t="inlineStr">
@@ -12543,54 +13891,54 @@
       </c>
       <c r="H145" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I145" s="4" t="inlineStr">
         <is>
-          <t>PASS, WARNING, NEEDS REVIEW</t>
+          <t>Sequential positive integers (1 to 330)</t>
         </is>
       </c>
       <c r="J145" s="4" t="inlineStr">
         <is>
-          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+          <t>Sequential institutional index for enumeration in the Pan-India census roster.</t>
         </is>
       </c>
       <c r="K145" s="4" t="inlineStr">
         <is>
-          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+          <t>Generated during census deduplication and synthesis.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NDC National Dental Colleges Register</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
         </is>
       </c>
       <c r="C146" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D146" s="9" t="inlineStr">
         <is>
-          <t>review_priority</t>
+          <t>Official ID</t>
         </is>
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F146" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="F146" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G146" s="5" t="inlineStr">
@@ -12600,44 +13948,44 @@
       </c>
       <c r="H146" s="4" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>409</t>
         </is>
       </c>
       <c r="I146" s="4" t="inlineStr">
         <is>
-          <t>HIGH, MEDIUM, LOW</t>
+          <t>Unique numeric string portal ID assigned by NDC/DCI</t>
         </is>
       </c>
       <c r="J146" s="4" t="inlineStr">
         <is>
-          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+          <t>Authoritative institutional identifier assigned by the National Dental Commission / Dental Council of India portal.</t>
         </is>
       </c>
       <c r="K146" s="4" t="inlineStr">
         <is>
-          <t>Calculated from quality_status and missing data thresholds.</t>
+          <t>Exposed in the College Search portal via SearchCollegeDetails.aspx?Id={id}. 100% unique.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NDC National Dental Colleges Register</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D147" s="9" t="inlineStr">
         <is>
-          <t>canonical_state</t>
+          <t>College Name</t>
         </is>
       </c>
       <c r="E147" s="5" t="inlineStr">
@@ -12645,9 +13993,9 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F147" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F147" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G147" s="5" t="inlineStr">
@@ -12657,44 +14005,44 @@
       </c>
       <c r="H147" s="4" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Anil Neerukonda Institute of Dental Sciences, Visakhapatnam</t>
         </is>
       </c>
       <c r="I147" s="4" t="inlineStr">
         <is>
-          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+          <t>Official registered dental institution title</t>
         </is>
       </c>
       <c r="J147" s="4" t="inlineStr">
         <is>
-          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+          <t>Full statutory name of the recognized dental college or institute.</t>
         </is>
       </c>
       <c r="K147" s="4" t="inlineStr">
         <is>
-          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+          <t>Extracted verbatim from the official College Search grid and detail page.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NDC National Dental Colleges Register</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
         </is>
       </c>
       <c r="C148" s="5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-27</t>
         </is>
       </c>
       <c r="D148" s="9" t="inlineStr">
         <is>
-          <t>inferred_district</t>
+          <t>State</t>
         </is>
       </c>
       <c r="E148" s="5" t="inlineStr">
@@ -12702,89 +14050,1742 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F148" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F148" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G148" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H148" s="4" t="inlineStr">
         <is>
-          <t>Ranga Reddy</t>
+          <t>Andhra Pradesh</t>
         </is>
       </c>
       <c r="I148" s="4" t="inlineStr">
         <is>
-          <t>Known Indian district name, or 'Not Specified'</t>
+          <t>Canonical Indian State or Union Territory name (28 States/UTs)</t>
         </is>
       </c>
       <c r="J148" s="4" t="inlineStr">
         <is>
-          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+          <t>State or Union Territory where the physical dental college campus is situated.</t>
         </is>
       </c>
       <c r="K148" s="4" t="inlineStr">
         <is>
-          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+          <t>Harmonized to the national census canonical 36 States/UTs reference catalog.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>District / City</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F149" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G149" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H149" s="4" t="inlineStr">
+        <is>
+          <t>Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="I149" s="4" t="inlineStr">
+        <is>
+          <t>District or municipality name, or 'PASS — SOURCE LIMITATION'</t>
+        </is>
+      </c>
+      <c r="J149" s="4" t="inlineStr">
+        <is>
+          <t>Official city or district location of the dental college campus.</t>
+        </is>
+      </c>
+      <c r="K149" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official detail page. Where absent in portal, marked 'PASS — SOURCE LIMITATION'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D150" s="9" t="inlineStr">
+        <is>
+          <t>PIN Code</t>
+        </is>
+      </c>
+      <c r="E150" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F150" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G150" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H150" s="4" t="inlineStr">
+        <is>
+          <t>531162</t>
+        </is>
+      </c>
+      <c r="I150" s="4" t="inlineStr">
+        <is>
+          <t>6-digit postal index number, or 'PASS — SOURCE LIMITATION'</t>
+        </is>
+      </c>
+      <c r="J150" s="4" t="inlineStr">
+        <is>
+          <t>Postal index number of the dental college campus.</t>
+        </is>
+      </c>
+      <c r="K150" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official college detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D151" s="9" t="inlineStr">
+        <is>
+          <t>Establishment Year</t>
+        </is>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F151" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G151" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H151" s="4" t="inlineStr">
+        <is>
+          <t>2013-14</t>
+        </is>
+      </c>
+      <c r="I151" s="4" t="inlineStr">
+        <is>
+          <t>Academic session or 4-digit calendar year (e.g. 1999-00, 2013-14)</t>
+        </is>
+      </c>
+      <c r="J151" s="4" t="inlineStr">
+        <is>
+          <t>Academic year in which the dental college was officially established and permitted.</t>
+        </is>
+      </c>
+      <c r="K151" s="4" t="inlineStr">
+        <is>
+          <t>Verified against official NDC College Search registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D152" s="9" t="inlineStr">
+        <is>
+          <t>Institution Type</t>
+        </is>
+      </c>
+      <c r="E152" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F152" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G152" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H152" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="I152" s="4" t="inlineStr">
+        <is>
+          <t>'Govt.', 'Private', 'Society', 'Trust', 'Autonomous'</t>
+        </is>
+      </c>
+      <c r="J152" s="4" t="inlineStr">
+        <is>
+          <t>Regulatory ownership and operational classification of the dental institution.</t>
+        </is>
+      </c>
+      <c r="K152" s="4" t="inlineStr">
+        <is>
+          <t>Captured directly from official DCI search table and detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D153" s="9" t="inlineStr">
+        <is>
+          <t>Management / Admin Authority</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F153" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G153" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H153" s="4" t="inlineStr">
+        <is>
+          <t>Society</t>
+        </is>
+      </c>
+      <c r="I153" s="4" t="inlineStr">
+        <is>
+          <t>'Society', 'Trust', 'Government', 'Autonomous', 'PASS — SOURCE LIMITATION'</t>
+        </is>
+      </c>
+      <c r="J153" s="4" t="inlineStr">
+        <is>
+          <t>Administrative authority, society, or trust running the dental institution.</t>
+        </is>
+      </c>
+      <c r="K153" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official institution detail record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>Affiliated University</t>
+        </is>
+      </c>
+      <c r="E154" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F154" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G154" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H154" s="4" t="inlineStr">
+        <is>
+          <t>Dr. N T R University of Health Sciences, Vijayawada</t>
+        </is>
+      </c>
+      <c r="I154" s="4" t="inlineStr">
+        <is>
+          <t>Name of affiliating health university, deemed university, or central institute</t>
+        </is>
+      </c>
+      <c r="J154" s="4" t="inlineStr">
+        <is>
+          <t>Statutory health sciences or general university to which the dental college is affiliated.</t>
+        </is>
+      </c>
+      <c r="K154" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official DCI affiliation schedule table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D155" s="9" t="inlineStr">
+        <is>
+          <t>Attached Hospital</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F155" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G155" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H155" s="4" t="inlineStr">
+        <is>
+          <t>Anil Neerukonda Hospital</t>
+        </is>
+      </c>
+      <c r="I155" s="4" t="inlineStr">
+        <is>
+          <t>Name of attached dental/general hospital or medical college</t>
+        </is>
+      </c>
+      <c r="J155" s="4" t="inlineStr">
+        <is>
+          <t>Teaching or general hospital attached to the dental college for clinical training.</t>
+        </is>
+      </c>
+      <c r="K155" s="4" t="inlineStr">
+        <is>
+          <t>Mandatory statutory requirement under NDC regulations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D156" s="9" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E156" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F156" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G156" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H156" s="4" t="inlineStr">
+        <is>
+          <t>Sangivalasa, visakhapatnam</t>
+        </is>
+      </c>
+      <c r="I156" s="4" t="inlineStr">
+        <is>
+          <t>Campus address lines or 'PASS — SOURCE LIMITATION'</t>
+        </is>
+      </c>
+      <c r="J156" s="4" t="inlineStr">
+        <is>
+          <t>Full street and campus location address lines.</t>
+        </is>
+      </c>
+      <c r="K156" s="4" t="inlineStr">
+        <is>
+          <t>Consolidated from Line 1 and Line 2 of official detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D157" s="9" t="inlineStr">
+        <is>
+          <t>BDS Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F157" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G157" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H157" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 100 seats</t>
+        </is>
+      </c>
+      <c r="I157" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats', 'Not Offered / None'</t>
+        </is>
+      </c>
+      <c r="J157" s="4" t="inlineStr">
+        <is>
+          <t>Undergraduate Bachelor of Dental Surgery (BDS) offering status and permitted intake capacity.</t>
+        </is>
+      </c>
+      <c r="K157" s="4" t="inlineStr">
+        <is>
+          <t>Synthesized from course-level records for AY 2026-27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D158" s="9" t="inlineStr">
+        <is>
+          <t>BDS Seats</t>
+        </is>
+      </c>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F158" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G158" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H158" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I158" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer (0, 40, 50, 60, 100)</t>
+        </is>
+      </c>
+      <c r="J158" s="4" t="inlineStr">
+        <is>
+          <t>Sanctioned annual undergraduate BDS student intake capacity.</t>
+        </is>
+      </c>
+      <c r="K158" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official College Search permitted seats table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D159" s="9" t="inlineStr">
+        <is>
+          <t>MDS Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F159" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G159" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H159" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 40 seats (9 specialities)</t>
+        </is>
+      </c>
+      <c r="I159" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats ({M} specialities)', 'Not Offered / None'</t>
+        </is>
+      </c>
+      <c r="J159" s="4" t="inlineStr">
+        <is>
+          <t>Postgraduate Master of Dental Surgery (MDS) status, total seats, and speciality diversity.</t>
+        </is>
+      </c>
+      <c r="K159" s="4" t="inlineStr">
+        <is>
+          <t>Aggregated from individual postgraduate speciality rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D160" s="9" t="inlineStr">
+        <is>
+          <t>MDS Seats</t>
+        </is>
+      </c>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F160" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G160" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H160" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I160" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer sum of all MDS speciality seats</t>
+        </is>
+      </c>
+      <c r="J160" s="4" t="inlineStr">
+        <is>
+          <t>Aggregate annual postgraduate MDS student intake capacity across all specialities.</t>
+        </is>
+      </c>
+      <c r="K160" s="4" t="inlineStr">
+        <is>
+          <t>Summed across all official MDS speciality allocations for AY 2026-27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D161" s="9" t="inlineStr">
+        <is>
+          <t>PG Diploma Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F161" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G161" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H161" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 3 seats (1 specialities)</t>
+        </is>
+      </c>
+      <c r="I161" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats ({M} specialities)', 'Not Offered / None'</t>
+        </is>
+      </c>
+      <c r="J161" s="4" t="inlineStr">
+        <is>
+          <t>Postgraduate Diploma course offering status and permitted intake capacity.</t>
+        </is>
+      </c>
+      <c r="K161" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from PG Diploma entries in official College Search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D162" s="9" t="inlineStr">
+        <is>
+          <t>PG Diploma Seats</t>
+        </is>
+      </c>
+      <c r="E162" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F162" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G162" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H162" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I162" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer (0, 1, 2, 3)</t>
+        </is>
+      </c>
+      <c r="J162" s="4" t="inlineStr">
+        <is>
+          <t>Total sanctioned PG Diploma seats at the institution.</t>
+        </is>
+      </c>
+      <c r="K162" s="4" t="inlineStr">
+        <is>
+          <t>Summed across all PG Diploma allocations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D163" s="9" t="inlineStr">
+        <is>
+          <t>DH Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F163" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G163" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H163" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 20 seats (Recognised)</t>
+        </is>
+      </c>
+      <c r="I163" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats (Recognised)', 'Not Offered / Not Listed'</t>
+        </is>
+      </c>
+      <c r="J163" s="4" t="inlineStr">
+        <is>
+          <t>Dental Hygienist (DH) diploma course recognition status and intake.</t>
+        </is>
+      </c>
+      <c r="K163" s="4" t="inlineStr">
+        <is>
+          <t>Matched from official NDC/DCI DH statutory schedule (DH.pdf).</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D164" s="9" t="inlineStr">
+        <is>
+          <t>DH Seats</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F164" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G164" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H164" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I164" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer (e.g. 0, 10, 20)</t>
+        </is>
+      </c>
+      <c r="J164" s="4" t="inlineStr">
+        <is>
+          <t>Sanctioned Dental Hygienist course capacity.</t>
+        </is>
+      </c>
+      <c r="K164" s="4" t="inlineStr">
+        <is>
+          <t>0 if not recognized/approved to run Dental Hygienists course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B165" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D165" s="9" t="inlineStr">
+        <is>
+          <t>DM Status &amp; Seats</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F165" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G165" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H165" s="4" t="inlineStr">
+        <is>
+          <t>Offered — 20 seats (Recognized)</t>
+        </is>
+      </c>
+      <c r="I165" s="4" t="inlineStr">
+        <is>
+          <t>'Offered — {N} seats (Recognized)', 'Not Offered / Not Listed'</t>
+        </is>
+      </c>
+      <c r="J165" s="4" t="inlineStr">
+        <is>
+          <t>Dental Mechanic (DM) diploma course recognition status and intake.</t>
+        </is>
+      </c>
+      <c r="K165" s="4" t="inlineStr">
+        <is>
+          <t>Matched from official NDC/DCI DM statutory schedule (DM.pdf).</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D166" s="9" t="inlineStr">
+        <is>
+          <t>DM Seats</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F166" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G166" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H166" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I166" s="4" t="inlineStr">
+        <is>
+          <t>Non-negative integer (e.g. 0, 10, 20)</t>
+        </is>
+      </c>
+      <c r="J166" s="4" t="inlineStr">
+        <is>
+          <t>Sanctioned Dental Mechanic course capacity.</t>
+        </is>
+      </c>
+      <c r="K166" s="4" t="inlineStr">
+        <is>
+          <t>0 if not recognized/approved to run Dental Mechanics course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D167" s="9" t="inlineStr">
+        <is>
+          <t>Total Dental Intake Capacity</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F167" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G167" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H167" s="4" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="I167" s="4" t="inlineStr">
+        <is>
+          <t>Sum of BDS, MDS, PG Diploma, DH, and DM seats</t>
+        </is>
+      </c>
+      <c r="J167" s="4" t="inlineStr">
+        <is>
+          <t>Total aggregate annual dental education student intake across all programs at the campus.</t>
+        </is>
+      </c>
+      <c r="K167" s="4" t="inlineStr">
+        <is>
+          <t>Calculated field: BDS Seats + MDS Seats + PG Diploma Seats + DH Seats + DM Seats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D168" s="9" t="inlineStr">
+        <is>
+          <t>Current Regulatory Status</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F168" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G168" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H168" s="4" t="inlineStr">
+        <is>
+          <t>Recognised / Permitted</t>
+        </is>
+      </c>
+      <c r="I168" s="4" t="inlineStr">
+        <is>
+          <t>'Recognised / Permitted', 'Recognition Withdrawn', 'Admissions Stopped', 'Permission Disapproved', 'Permitted (Seats Reduced / Surrendered)', 'Permitted (Court Order / Sub-Judice)', 'Recognised / Permitted (Seats Revised)', 'Conditional / Regulatory Remark Noted'</t>
+        </is>
+      </c>
+      <c r="J168" s="4" t="inlineStr">
+        <is>
+          <t>Harmonized regulatory approval and operational status under the NDC Act, 2023.</t>
+        </is>
+      </c>
+      <c r="K168" s="4" t="inlineStr">
+        <is>
+          <t>Synthesized directly from official portal remarks without dropping any restricted institutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D169" s="9" t="inlineStr">
+        <is>
+          <t>Regulatory Remarks</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F169" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G169" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H169" s="4" t="inlineStr">
+        <is>
+          <t>No adverse remarks on record</t>
+        </is>
+      </c>
+      <c r="I169" s="4" t="inlineStr">
+        <is>
+          <t>Full verbatim regulatory note, or 'No adverse remarks on record'</t>
+        </is>
+      </c>
+      <c r="J169" s="4" t="inlineStr">
+        <is>
+          <t>Verbatim statutory remarks, court orders, seat reduction directives, or withdrawal notices.</t>
+        </is>
+      </c>
+      <c r="K169" s="4" t="inlineStr">
+        <is>
+          <t>Captured directly from the official portal's Remark column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D170" s="9" t="inlineStr">
+        <is>
+          <t>Official Detail URL</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="F170" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G170" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H170" s="4" t="inlineStr">
+        <is>
+          <t>https://dciindia.gov.in/SearchCollegeDetails.aspx?Id=409</t>
+        </is>
+      </c>
+      <c r="I170" s="4" t="inlineStr">
+        <is>
+          <t>Official detail page URL on dciindia.gov.in</t>
+        </is>
+      </c>
+      <c r="J170" s="4" t="inlineStr">
+        <is>
+          <t>Direct clickable link to the official college profile on the NDC/DCI portal.</t>
+        </is>
+      </c>
+      <c r="K170" s="4" t="inlineStr">
+        <is>
+          <t>Preserves audit trail and public provenance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B171" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D171" s="9" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="F171" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G171" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H171" s="4" t="inlineStr">
+        <is>
+          <t>https://dciindia.gov.in/CollegeSearch.aspx</t>
+        </is>
+      </c>
+      <c r="I171" s="4" t="inlineStr">
+        <is>
+          <t>https://dciindia.gov.in/CollegeSearch.aspx</t>
+        </is>
+      </c>
+      <c r="J171" s="4" t="inlineStr">
+        <is>
+          <t>Authoritative primary source URL from which the national institutional data was harvested.</t>
+        </is>
+      </c>
+      <c r="K171" s="4" t="inlineStr">
+        <is>
+          <t>Census primary source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D172" s="9" t="inlineStr">
+        <is>
+          <t>Academic Year</t>
+        </is>
+      </c>
+      <c r="E172" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F172" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G172" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H172" s="4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="I172" s="4" t="inlineStr">
+        <is>
+          <t>'2026-27'</t>
+        </is>
+      </c>
+      <c r="J172" s="4" t="inlineStr">
+        <is>
+          <t>Official regulatory academic session to which the permission and seat matrix applies.</t>
+        </is>
+      </c>
+      <c r="K172" s="4" t="inlineStr">
+        <is>
+          <t>Standardized to official NDC session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="4" t="inlineStr">
+        <is>
+          <t>NDC National Dental Colleges Register</t>
+        </is>
+      </c>
+      <c r="B173" s="4" t="inlineStr">
+        <is>
+          <t>National Dental Commission (NDC) / former Dental Council of India (DCI)</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="D173" s="9" t="inlineStr">
+        <is>
+          <t>Collection Date</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F173" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G173" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H173" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I173" s="4" t="inlineStr">
+        <is>
+          <t>ISO 8601 Date (YYYY-MM-DD)</t>
+        </is>
+      </c>
+      <c r="J173" s="4" t="inlineStr">
+        <is>
+          <t>Date when the official NDC national college dataset was extracted.</t>
+        </is>
+      </c>
+      <c r="K173" s="4" t="inlineStr">
+        <is>
+          <t>Timestamp of census compilation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="4" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B149" s="4" t="inlineStr">
+      <c r="B174" s="4" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C149" s="5" t="inlineStr">
+      <c r="C174" s="5" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D149" s="9" t="inlineStr">
+      <c r="D174" s="9" t="inlineStr">
+        <is>
+          <t>quality_status</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F174" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G174" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H174" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I174" s="4" t="inlineStr">
+        <is>
+          <t>PASS, WARNING, NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="J174" s="4" t="inlineStr">
+        <is>
+          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+        </is>
+      </c>
+      <c r="K174" s="4" t="inlineStr">
+        <is>
+          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B175" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D175" s="9" t="inlineStr">
+        <is>
+          <t>review_priority</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F175" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G175" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H175" s="4" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I175" s="4" t="inlineStr">
+        <is>
+          <t>HIGH, MEDIUM, LOW</t>
+        </is>
+      </c>
+      <c r="J175" s="4" t="inlineStr">
+        <is>
+          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+        </is>
+      </c>
+      <c r="K175" s="4" t="inlineStr">
+        <is>
+          <t>Calculated from quality_status and missing data thresholds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D176" s="9" t="inlineStr">
+        <is>
+          <t>canonical_state</t>
+        </is>
+      </c>
+      <c r="E176" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F176" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G176" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H176" s="4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="I176" s="4" t="inlineStr">
+        <is>
+          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+        </is>
+      </c>
+      <c r="J176" s="4" t="inlineStr">
+        <is>
+          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+        </is>
+      </c>
+      <c r="K176" s="4" t="inlineStr">
+        <is>
+          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D177" s="9" t="inlineStr">
+        <is>
+          <t>inferred_district</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F177" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G177" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H177" s="4" t="inlineStr">
+        <is>
+          <t>Ranga Reddy</t>
+        </is>
+      </c>
+      <c r="I177" s="4" t="inlineStr">
+        <is>
+          <t>Known Indian district name, or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="J177" s="4" t="inlineStr">
+        <is>
+          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+        </is>
+      </c>
+      <c r="K177" s="4" t="inlineStr">
+        <is>
+          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D178" s="9" t="inlineStr">
         <is>
           <t>_search_blob</t>
         </is>
       </c>
-      <c r="E149" s="5" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F149" s="12" t="inlineStr">
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F178" s="12" t="inlineStr">
         <is>
           <t>DASHBOARD-CALCULATED FIELD</t>
         </is>
       </c>
-      <c r="G149" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H149" s="4" t="inlineStr">
+      <c r="G178" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H178" s="4" t="inlineStr">
         <is>
           <t>iiit hyderabad international institute of information technology gachibowli telangana 500032</t>
         </is>
       </c>
-      <c r="I149" s="4" t="inlineStr">
+      <c r="I178" s="4" t="inlineStr">
         <is>
           <t>Lowercase normalized concatenated search token string</t>
         </is>
       </c>
-      <c r="J149" s="4" t="inlineStr">
+      <c r="J178" s="4" t="inlineStr">
         <is>
           <t>Unified multi-attribute token string combining Name, State, District, Address, PIN, ID, University, and Locality Aliases for fast sub-millisecond global search.</t>
         </is>
       </c>
-      <c r="K149" s="4" t="inlineStr">
+      <c r="K178" s="4" t="inlineStr">
         <is>
           <t>Powers /api/search and in-table search across all 7,335 final list records.</t>
         </is>

</xml_diff>

<commit_message>
Add official NCTE teacher education dataset and update category colors
</commit_message>
<xml_diff>
--- a/DATA_DICTIONARY.xlsx
+++ b/DATA_DICTIONARY.xlsx
@@ -22,7 +22,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NCH_Homoeopathy" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCI_Law" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDC_Dental" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Calculated" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NCTE_Teacher" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Calculated" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -533,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1394,53 +1395,108 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Teacher Education (B.Ed / D.El.Ed / M.Ed / B.P.Ed / ITEP / etc.)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>17,556</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>35 / 36 (97%)</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>NCTE Institute ID (e.g. NCTE1410672)</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education Official Portal &amp; Regional Committee Rosters (ERC, NRC, SRC, WRC)</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>100% complete national census of recognized teacher education institutions across India under NCTE Act, 1993. Multi-course offerings mapped to dedicated Programmes &amp; Courses catalog (28,372 entries), and 1,274 withdrawn/de-recognized institutions isolated in dedicated audit registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Cross-Cutting Metadata &amp; Search</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>10,708 Final Records</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>36 / 36 (100%)</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>N/A (Derived Attributes)</t>
         </is>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="I20" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>Pan-India Data Quality &amp; Deduplication Engine</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Standardized canonical state, inferred district, quality status, and search blobs.</t>
         </is>
@@ -5345,6 +5401,962 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DATA DICTIONARY: NCTE NATIONAL TEACHER EDUCATION COLLEGES REGISTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Field / Column Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Field Classification</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Required?</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Example Value</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Allowed Values / Codebook</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Description / Meaning</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Methodological Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Sequential positive integers (1 to 17,556)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Sequential institutional index for enumeration in the Pan-India census roster.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Generated during census deduplication and synthesis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>NCTE Institute ID</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>NCTE1410672</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Alphanumeric string prefix NCTE + numeric identifier</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Authoritative institutional identifier assigned by National Council for Teacher Education portal.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Primary key uniquely identifying each physical campus. 100% unique across the roster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Institution Name</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Arunachal University of Studies</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Official statutory institution name</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Full statutory name of the recognized teacher education college or university department.</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Verbatim from official NCTE portal registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Arunachal Pradesh</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>36 Standard States and Union Territories</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>State or Union Territory where the physical teacher education campus is situated.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Harmonized to the national census canonical 36 States/UTs catalog across 4 Regional Committees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Lohit</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>District name or 'Unassigned'</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Administrative district location of the institution campus.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official NCTE portal listings; where not specified in portal, labeled 'Unassigned'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>PIN Code</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>792103</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>6-digit postal code or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Postal index number of the institution campus.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from registered campus address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Vill - Deobeel, Street/Road - NH-52, Taluka/Mandal - Namsai</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Postal address text or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Complete statutory physical premises address of the teacher education institution.</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Preserved from official NCTE regulatory records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Management Type</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Private Institution</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Government / Private / University / Self-Financed / Constituent</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Statutory management and governance classification of the institution.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Official NCTE management classification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Affiliating University</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Rajiv Gandhi University</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Name of affiliating state/central university or board</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Statutory examining body or university to which the teacher education programmes are affiliated.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Official affiliating body declared in NCTE recognition records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Regional Committee</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>ERC</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>ERC, NRC, SRC, WRC</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>NCTE Regional Committee holding statutory jurisdiction (Eastern, Northern, Southern, or Western).</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>ERC (Eastern), NRC (Northern), SRC (Southern), WRC (Western).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Recognition Status</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Recognized</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Recognized / Permitted</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Current legal regulatory recognition status under the NCTE Act, 1993.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>All 17,556 institutions in this roster are active recognized entities. Withdrawn institutions are maintained in a separate sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Recognized Programmes</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>B.Ed, D.El.Ed, M.Ed</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Comma-separated list of recognized teacher education course names</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Summary of all recognized professional education programmes offered at this physical campus.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Aggregated across all official recognition orders for this campus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Total Approved Intake</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Total sanctioned annual intake (seats) or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Combined total annual student intake approved by NCTE across all active recognized courses at this institution.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Summed across all recognized course orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Total Recognized Courses</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Positive integer (e.g. 1, 2, 3...)</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Total number of distinct NCTE-approved academic programmes/units operating at this campus.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Calculated from institutional programme breakdown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Latest Applicable Session</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>2017-2018</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Academic session string (e.g. 2019-2020, 2026-27)</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Latest regulatory academic session or order revision year recorded by NCTE.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official order details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Contact Number</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>0380-6202797 / 9540542220</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Telephone/mobile number string</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Official institutional telephone or mobile contact number.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>As published on official NCTE portal directory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>registrar@arunachaluniversity.ac.in</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Valid email address format</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Official institutional contact email address.</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>As published on official NCTE portal directory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>www.arunachaluniversity.ac.in</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Web URL domain</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Official website URL of the teacher education institution.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>As published on official NCTE portal directory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Official Source Portal</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>NCTE Official Portal (web.ncte.gov.in)</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Authoritative portal label</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Designated official government regulatory portal providing the statutory data.</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education statutory web portal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>https://web.ncte.gov.in/page-regional-committee-institution-lists/3/arunachal-pradesh</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Valid HTTP/HTTPS URL</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Direct official URL endpoint where the state institutional list is published.</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Traceable source endpoint for regulatory auditing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Collection Date</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD date format</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Date on which the institutional record was retrieved from the official NCTE portal.</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Timestamp of the census crawling pass.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5629,7 +6641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K178"/>
+  <dimension ref="A1:K199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -15509,12 +16521,12 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NCTE National Teacher Education Colleges Register</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Council for Teacher Education (NCTE)</t>
         </is>
       </c>
       <c r="C174" s="5" t="inlineStr">
@@ -15524,17 +16536,17 @@
       </c>
       <c r="D174" s="9" t="inlineStr">
         <is>
-          <t>quality_status</t>
+          <t>S.No</t>
         </is>
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F174" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F174" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
         </is>
       </c>
       <c r="G174" s="5" t="inlineStr">
@@ -15544,34 +16556,34 @@
       </c>
       <c r="H174" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I174" s="4" t="inlineStr">
         <is>
-          <t>PASS, WARNING, NEEDS REVIEW</t>
+          <t>Sequential positive integers (1 to 17,556)</t>
         </is>
       </c>
       <c r="J174" s="4" t="inlineStr">
         <is>
-          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+          <t>Sequential institutional index for enumeration in the Pan-India census roster.</t>
         </is>
       </c>
       <c r="K174" s="4" t="inlineStr">
         <is>
-          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+          <t>Generated during census deduplication and synthesis.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NCTE National Teacher Education Colleges Register</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Council for Teacher Education (NCTE)</t>
         </is>
       </c>
       <c r="C175" s="5" t="inlineStr">
@@ -15581,17 +16593,17 @@
       </c>
       <c r="D175" s="9" t="inlineStr">
         <is>
-          <t>review_priority</t>
+          <t>NCTE Institute ID</t>
         </is>
       </c>
       <c r="E175" s="5" t="inlineStr">
         <is>
-          <t>String (Categorical)</t>
-        </is>
-      </c>
-      <c r="F175" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F175" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G175" s="5" t="inlineStr">
@@ -15601,34 +16613,34 @@
       </c>
       <c r="H175" s="4" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>NCTE1410672</t>
         </is>
       </c>
       <c r="I175" s="4" t="inlineStr">
         <is>
-          <t>HIGH, MEDIUM, LOW</t>
+          <t>Alphanumeric string prefix NCTE + numeric identifier</t>
         </is>
       </c>
       <c r="J175" s="4" t="inlineStr">
         <is>
-          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+          <t>Authoritative institutional identifier assigned by National Council for Teacher Education portal.</t>
         </is>
       </c>
       <c r="K175" s="4" t="inlineStr">
         <is>
-          <t>Calculated from quality_status and missing data thresholds.</t>
+          <t>Primary key uniquely identifying each physical campus. 100% unique across the roster.</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NCTE National Teacher Education Colleges Register</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Council for Teacher Education (NCTE)</t>
         </is>
       </c>
       <c r="C176" s="5" t="inlineStr">
@@ -15638,7 +16650,7 @@
       </c>
       <c r="D176" s="9" t="inlineStr">
         <is>
-          <t>canonical_state</t>
+          <t>Institution Name</t>
         </is>
       </c>
       <c r="E176" s="5" t="inlineStr">
@@ -15646,9 +16658,9 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F176" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F176" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G176" s="5" t="inlineStr">
@@ -15658,34 +16670,34 @@
       </c>
       <c r="H176" s="4" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Arunachal University of Studies</t>
         </is>
       </c>
       <c r="I176" s="4" t="inlineStr">
         <is>
-          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+          <t>Official statutory institution name</t>
         </is>
       </c>
       <c r="J176" s="4" t="inlineStr">
         <is>
-          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+          <t>Full statutory name of the recognized teacher education college or university department.</t>
         </is>
       </c>
       <c r="K176" s="4" t="inlineStr">
         <is>
-          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+          <t>Verbatim from official NCTE portal registry.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>Dashboard Common Architecture</t>
+          <t>NCTE National Teacher Education Colleges Register</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>National Census Dashboard Engine</t>
+          <t>National Council for Teacher Education (NCTE)</t>
         </is>
       </c>
       <c r="C177" s="5" t="inlineStr">
@@ -15695,7 +16707,7 @@
       </c>
       <c r="D177" s="9" t="inlineStr">
         <is>
-          <t>inferred_district</t>
+          <t>State</t>
         </is>
       </c>
       <c r="E177" s="5" t="inlineStr">
@@ -15703,89 +16715,1286 @@
           <t>String</t>
         </is>
       </c>
-      <c r="F177" s="12" t="inlineStr">
-        <is>
-          <t>DASHBOARD-CALCULATED FIELD</t>
+      <c r="F177" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
         </is>
       </c>
       <c r="G177" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H177" s="4" t="inlineStr">
         <is>
-          <t>Ranga Reddy</t>
+          <t>Arunachal Pradesh</t>
         </is>
       </c>
       <c r="I177" s="4" t="inlineStr">
         <is>
-          <t>Known Indian district name, or 'Not Specified'</t>
+          <t>36 Standard States and Union Territories</t>
         </is>
       </c>
       <c r="J177" s="4" t="inlineStr">
         <is>
-          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+          <t>State or Union Territory where the physical teacher education campus is situated.</t>
         </is>
       </c>
       <c r="K177" s="4" t="inlineStr">
         <is>
-          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+          <t>Harmonized to the national census canonical 36 States/UTs catalog across 4 Regional Committees.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D178" s="9" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F178" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G178" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H178" s="4" t="inlineStr">
+        <is>
+          <t>Lohit</t>
+        </is>
+      </c>
+      <c r="I178" s="4" t="inlineStr">
+        <is>
+          <t>District name or 'Unassigned'</t>
+        </is>
+      </c>
+      <c r="J178" s="4" t="inlineStr">
+        <is>
+          <t>Administrative district location of the institution campus.</t>
+        </is>
+      </c>
+      <c r="K178" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official NCTE portal listings; where not specified in portal, labeled 'Unassigned'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D179" s="9" t="inlineStr">
+        <is>
+          <t>PIN Code</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F179" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G179" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H179" s="4" t="inlineStr">
+        <is>
+          <t>792103</t>
+        </is>
+      </c>
+      <c r="I179" s="4" t="inlineStr">
+        <is>
+          <t>6-digit postal code or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="J179" s="4" t="inlineStr">
+        <is>
+          <t>Postal index number of the institution campus.</t>
+        </is>
+      </c>
+      <c r="K179" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from registered campus address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D180" s="9" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E180" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F180" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G180" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H180" s="4" t="inlineStr">
+        <is>
+          <t>Vill - Deobeel, Street/Road - NH-52, Taluka/Mandal - Namsai</t>
+        </is>
+      </c>
+      <c r="I180" s="4" t="inlineStr">
+        <is>
+          <t>Postal address text or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="J180" s="4" t="inlineStr">
+        <is>
+          <t>Complete statutory physical premises address of the teacher education institution.</t>
+        </is>
+      </c>
+      <c r="K180" s="4" t="inlineStr">
+        <is>
+          <t>Preserved from official NCTE regulatory records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D181" s="9" t="inlineStr">
+        <is>
+          <t>Management Type</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F181" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G181" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H181" s="4" t="inlineStr">
+        <is>
+          <t>Private Institution</t>
+        </is>
+      </c>
+      <c r="I181" s="4" t="inlineStr">
+        <is>
+          <t>Government / Private / University / Self-Financed / Constituent</t>
+        </is>
+      </c>
+      <c r="J181" s="4" t="inlineStr">
+        <is>
+          <t>Statutory management and governance classification of the institution.</t>
+        </is>
+      </c>
+      <c r="K181" s="4" t="inlineStr">
+        <is>
+          <t>Official NCTE management classification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D182" s="9" t="inlineStr">
+        <is>
+          <t>Affiliating University</t>
+        </is>
+      </c>
+      <c r="E182" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F182" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G182" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H182" s="4" t="inlineStr">
+        <is>
+          <t>Rajiv Gandhi University</t>
+        </is>
+      </c>
+      <c r="I182" s="4" t="inlineStr">
+        <is>
+          <t>Name of affiliating state/central university or board</t>
+        </is>
+      </c>
+      <c r="J182" s="4" t="inlineStr">
+        <is>
+          <t>Statutory examining body or university to which the teacher education programmes are affiliated.</t>
+        </is>
+      </c>
+      <c r="K182" s="4" t="inlineStr">
+        <is>
+          <t>Official affiliating body declared in NCTE recognition records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D183" s="9" t="inlineStr">
+        <is>
+          <t>Regional Committee</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F183" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G183" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H183" s="4" t="inlineStr">
+        <is>
+          <t>ERC</t>
+        </is>
+      </c>
+      <c r="I183" s="4" t="inlineStr">
+        <is>
+          <t>ERC, NRC, SRC, WRC</t>
+        </is>
+      </c>
+      <c r="J183" s="4" t="inlineStr">
+        <is>
+          <t>NCTE Regional Committee holding statutory jurisdiction (Eastern, Northern, Southern, or Western).</t>
+        </is>
+      </c>
+      <c r="K183" s="4" t="inlineStr">
+        <is>
+          <t>ERC (Eastern), NRC (Northern), SRC (Southern), WRC (Western).</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D184" s="9" t="inlineStr">
+        <is>
+          <t>Recognition Status</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F184" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G184" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H184" s="4" t="inlineStr">
+        <is>
+          <t>Recognized</t>
+        </is>
+      </c>
+      <c r="I184" s="4" t="inlineStr">
+        <is>
+          <t>Recognized / Permitted</t>
+        </is>
+      </c>
+      <c r="J184" s="4" t="inlineStr">
+        <is>
+          <t>Current legal regulatory recognition status under the NCTE Act, 1993.</t>
+        </is>
+      </c>
+      <c r="K184" s="4" t="inlineStr">
+        <is>
+          <t>All 17,556 institutions in this roster are active recognized entities. Withdrawn institutions are maintained in a separate sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D185" s="9" t="inlineStr">
+        <is>
+          <t>Recognized Programmes</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F185" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H185" s="4" t="inlineStr">
+        <is>
+          <t>B.Ed, D.El.Ed, M.Ed</t>
+        </is>
+      </c>
+      <c r="I185" s="4" t="inlineStr">
+        <is>
+          <t>Comma-separated list of recognized teacher education course names</t>
+        </is>
+      </c>
+      <c r="J185" s="4" t="inlineStr">
+        <is>
+          <t>Summary of all recognized professional education programmes offered at this physical campus.</t>
+        </is>
+      </c>
+      <c r="K185" s="4" t="inlineStr">
+        <is>
+          <t>Aggregated across all official recognition orders for this campus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D186" s="9" t="inlineStr">
+        <is>
+          <t>Total Approved Intake</t>
+        </is>
+      </c>
+      <c r="E186" s="5" t="inlineStr">
+        <is>
+          <t>Integer (String)</t>
+        </is>
+      </c>
+      <c r="F186" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G186" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H186" s="4" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="I186" s="4" t="inlineStr">
+        <is>
+          <t>Total sanctioned annual intake (seats) or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="J186" s="4" t="inlineStr">
+        <is>
+          <t>Combined total annual student intake approved by NCTE across all active recognized courses at this institution.</t>
+        </is>
+      </c>
+      <c r="K186" s="4" t="inlineStr">
+        <is>
+          <t>Summed across all recognized course orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D187" s="9" t="inlineStr">
+        <is>
+          <t>Total Recognized Courses</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="F187" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H187" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I187" s="4" t="inlineStr">
+        <is>
+          <t>Positive integer (e.g. 1, 2, 3...)</t>
+        </is>
+      </c>
+      <c r="J187" s="4" t="inlineStr">
+        <is>
+          <t>Total number of distinct NCTE-approved academic programmes/units operating at this campus.</t>
+        </is>
+      </c>
+      <c r="K187" s="4" t="inlineStr">
+        <is>
+          <t>Calculated from institutional programme breakdown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D188" s="9" t="inlineStr">
+        <is>
+          <t>Latest Applicable Session</t>
+        </is>
+      </c>
+      <c r="E188" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F188" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G188" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H188" s="4" t="inlineStr">
+        <is>
+          <t>2017-2018</t>
+        </is>
+      </c>
+      <c r="I188" s="4" t="inlineStr">
+        <is>
+          <t>Academic session string (e.g. 2019-2020, 2026-27)</t>
+        </is>
+      </c>
+      <c r="J188" s="4" t="inlineStr">
+        <is>
+          <t>Latest regulatory academic session or order revision year recorded by NCTE.</t>
+        </is>
+      </c>
+      <c r="K188" s="4" t="inlineStr">
+        <is>
+          <t>Extracted from official order details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D189" s="9" t="inlineStr">
+        <is>
+          <t>Contact Number</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F189" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G189" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H189" s="4" t="inlineStr">
+        <is>
+          <t>0380-6202797 / 9540542220</t>
+        </is>
+      </c>
+      <c r="I189" s="4" t="inlineStr">
+        <is>
+          <t>Telephone/mobile number string</t>
+        </is>
+      </c>
+      <c r="J189" s="4" t="inlineStr">
+        <is>
+          <t>Official institutional telephone or mobile contact number.</t>
+        </is>
+      </c>
+      <c r="K189" s="4" t="inlineStr">
+        <is>
+          <t>As published on official NCTE portal directory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D190" s="9" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E190" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F190" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G190" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H190" s="4" t="inlineStr">
+        <is>
+          <t>registrar@arunachaluniversity.ac.in</t>
+        </is>
+      </c>
+      <c r="I190" s="4" t="inlineStr">
+        <is>
+          <t>Valid email address format</t>
+        </is>
+      </c>
+      <c r="J190" s="4" t="inlineStr">
+        <is>
+          <t>Official institutional contact email address.</t>
+        </is>
+      </c>
+      <c r="K190" s="4" t="inlineStr">
+        <is>
+          <t>As published on official NCTE portal directory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D191" s="9" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F191" s="10" t="inlineStr">
+        <is>
+          <t>SOURCE FIELD</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H191" s="4" t="inlineStr">
+        <is>
+          <t>www.arunachaluniversity.ac.in</t>
+        </is>
+      </c>
+      <c r="I191" s="4" t="inlineStr">
+        <is>
+          <t>Web URL domain</t>
+        </is>
+      </c>
+      <c r="J191" s="4" t="inlineStr">
+        <is>
+          <t>Official website URL of the teacher education institution.</t>
+        </is>
+      </c>
+      <c r="K191" s="4" t="inlineStr">
+        <is>
+          <t>As published on official NCTE portal directory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D192" s="9" t="inlineStr">
+        <is>
+          <t>Official Source Portal</t>
+        </is>
+      </c>
+      <c r="E192" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F192" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G192" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H192" s="4" t="inlineStr">
+        <is>
+          <t>NCTE Official Portal (web.ncte.gov.in)</t>
+        </is>
+      </c>
+      <c r="I192" s="4" t="inlineStr">
+        <is>
+          <t>Authoritative portal label</t>
+        </is>
+      </c>
+      <c r="J192" s="4" t="inlineStr">
+        <is>
+          <t>Designated official government regulatory portal providing the statutory data.</t>
+        </is>
+      </c>
+      <c r="K192" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education statutory web portal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D193" s="9" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F193" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H193" s="4" t="inlineStr">
+        <is>
+          <t>https://web.ncte.gov.in/page-regional-committee-institution-lists/3/arunachal-pradesh</t>
+        </is>
+      </c>
+      <c r="I193" s="4" t="inlineStr">
+        <is>
+          <t>Valid HTTP/HTTPS URL</t>
+        </is>
+      </c>
+      <c r="J193" s="4" t="inlineStr">
+        <is>
+          <t>Direct official URL endpoint where the state institutional list is published.</t>
+        </is>
+      </c>
+      <c r="K193" s="4" t="inlineStr">
+        <is>
+          <t>Traceable source endpoint for regulatory auditing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>NCTE National Teacher Education Colleges Register</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>National Council for Teacher Education (NCTE)</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D194" s="9" t="inlineStr">
+        <is>
+          <t>Collection Date</t>
+        </is>
+      </c>
+      <c r="E194" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F194" s="11" t="inlineStr">
+        <is>
+          <t>DERIVED FIELD</t>
+        </is>
+      </c>
+      <c r="G194" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H194" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I194" s="4" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD date format</t>
+        </is>
+      </c>
+      <c r="J194" s="4" t="inlineStr">
+        <is>
+          <t>Date on which the institutional record was retrieved from the official NCTE portal.</t>
+        </is>
+      </c>
+      <c r="K194" s="4" t="inlineStr">
+        <is>
+          <t>Timestamp of the census crawling pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B178" s="4" t="inlineStr">
+      <c r="B195" s="4" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C178" s="5" t="inlineStr">
+      <c r="C195" s="5" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D178" s="9" t="inlineStr">
+      <c r="D195" s="9" t="inlineStr">
+        <is>
+          <t>quality_status</t>
+        </is>
+      </c>
+      <c r="E195" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F195" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G195" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H195" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I195" s="4" t="inlineStr">
+        <is>
+          <t>PASS, WARNING, NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="J195" s="4" t="inlineStr">
+        <is>
+          <t>Automated data quality score computed by inspecting name completeness, state tagging rate, and official regulatory ID duplication.</t>
+        </is>
+      </c>
+      <c r="K195" s="4" t="inlineStr">
+        <is>
+          <t>Calculated by DataRegistry._analyze_dataframe() on server startup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C196" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D196" s="9" t="inlineStr">
+        <is>
+          <t>review_priority</t>
+        </is>
+      </c>
+      <c r="E196" s="5" t="inlineStr">
+        <is>
+          <t>String (Categorical)</t>
+        </is>
+      </c>
+      <c r="F196" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G196" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H196" s="4" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I196" s="4" t="inlineStr">
+        <is>
+          <t>HIGH, MEDIUM, LOW</t>
+        </is>
+      </c>
+      <c r="J196" s="4" t="inlineStr">
+        <is>
+          <t>Executive triage priority assigned to guide research team attention toward datasets with missing attributes or pending deduplication.</t>
+        </is>
+      </c>
+      <c r="K196" s="4" t="inlineStr">
+        <is>
+          <t>Calculated from quality_status and missing data thresholds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B197" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D197" s="9" t="inlineStr">
+        <is>
+          <t>canonical_state</t>
+        </is>
+      </c>
+      <c r="E197" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F197" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G197" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H197" s="4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="I197" s="4" t="inlineStr">
+        <is>
+          <t>One of 36 Canonical States &amp; UTs, or 'Unknown / Unclassified'</t>
+        </is>
+      </c>
+      <c r="J197" s="4" t="inlineStr">
+        <is>
+          <t>Standardized State or Union Territory name produced by passing raw state strings through STATE_SYNONYMS and CANONICAL_LOWER_MAP.</t>
+        </is>
+      </c>
+      <c r="K197" s="4" t="inlineStr">
+        <is>
+          <t>Enforces 100% canonical state aggregation without duplicate state spelling variants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D198" s="9" t="inlineStr">
+        <is>
+          <t>inferred_district</t>
+        </is>
+      </c>
+      <c r="E198" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F198" s="12" t="inlineStr">
+        <is>
+          <t>DASHBOARD-CALCULATED FIELD</t>
+        </is>
+      </c>
+      <c r="G198" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H198" s="4" t="inlineStr">
+        <is>
+          <t>Ranga Reddy</t>
+        </is>
+      </c>
+      <c r="I198" s="4" t="inlineStr">
+        <is>
+          <t>Known Indian district name, or 'Not Specified'</t>
+        </is>
+      </c>
+      <c r="J198" s="4" t="inlineStr">
+        <is>
+          <t>District name inferred by regex scanning of full address and locality strings when explicit district column is missing or null.</t>
+        </is>
+      </c>
+      <c r="K198" s="4" t="inlineStr">
+        <is>
+          <t>Computed by extract_district_from_address() using KNOWN_DISTRICTS catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard Common Architecture</t>
+        </is>
+      </c>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>National Census Dashboard Engine</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D199" s="9" t="inlineStr">
         <is>
           <t>_search_blob</t>
         </is>
       </c>
-      <c r="E178" s="5" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="F178" s="12" t="inlineStr">
+      <c r="E199" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F199" s="12" t="inlineStr">
         <is>
           <t>DASHBOARD-CALCULATED FIELD</t>
         </is>
       </c>
-      <c r="G178" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H178" s="4" t="inlineStr">
+      <c r="G199" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H199" s="4" t="inlineStr">
         <is>
           <t>iiit hyderabad international institute of information technology gachibowli telangana 500032</t>
         </is>
       </c>
-      <c r="I178" s="4" t="inlineStr">
+      <c r="I199" s="4" t="inlineStr">
         <is>
           <t>Lowercase normalized concatenated search token string</t>
         </is>
       </c>
-      <c r="J178" s="4" t="inlineStr">
+      <c r="J199" s="4" t="inlineStr">
         <is>
           <t>Unified multi-attribute token string combining Name, State, District, Address, PIN, ID, University, and Locality Aliases for fast sub-millisecond global search.</t>
         </is>
       </c>
-      <c r="K178" s="4" t="inlineStr">
+      <c r="K199" s="4" t="inlineStr">
         <is>
           <t>Powers /api/search and in-table search across all 7,335 final list records.</t>
         </is>

</xml_diff>

<commit_message>
feat(icar): extract, validate and integrate ICAR agricultural institutions dataset (159 canonical institutions, 1347 programmes across 23 States/UTs)
</commit_message>
<xml_diff>
--- a/DATA_DICTIONARY.xlsx
+++ b/DATA_DICTIONARY.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="48" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
@@ -1450,53 +1450,163 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
+          <t>VCI National Veterinary Colleges Register</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Veterinary Council of India (VCI) / DAHD</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Veterinary Sciences (B.V.Sc &amp; A.H.)</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>26 / 36 (72%)</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Registration / VCI Code (VCI Canonical ID)</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>Indian Veterinary Council Act, 1984 Gazette Rosters</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>100% complete national census of 96 canonical physical veterinary institutions (72 Recognized, 24 Provisionally Recognized) across India.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>ICAR Agricultural &amp; Allied Institutions Register</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Indian Council of Agricultural Research (ICAR)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Agricultural &amp; Allied Sciences</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>2024-26</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>159</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>23 / 36 (64%)</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>ICAR_Serial</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>ICAR National Agricultural Education Accreditation Board (NAEAB) Official Circular Lists (List 1, 1A, 2, 3)</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>100% complete national census of 159 canonical ICAR-accredited agricultural institutions and 1,347 accredited degree programmes across India.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
           <t>Dashboard Common Architecture</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>National Census Dashboard Engine</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Cross-Cutting Metadata &amp; Search</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>10,708 Final Records</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>36 / 36 (100%)</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>N/A (Derived Attributes)</t>
         </is>
       </c>
-      <c r="I20" s="7" t="n">
+      <c r="I22" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Pan-India Data Quality &amp; Deduplication Engine</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>Standardized canonical state, inferred district, quality status, and search blobs.</t>
         </is>

</xml_diff>